<commit_message>
codeableconcept text is set to null if empty. practitioner identifier added
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mriley7\workspace\raven-import-and-submit-api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE25A5C-6F17-4CFF-ADB6-752314F8A397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF75D8B1-DCC4-0240-A3D0-DC3970BA3F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Base Input Schema" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="218">
   <si>
     <t>Sections</t>
   </si>
@@ -906,6 +906,14 @@
   </si>
   <si>
     <t>Full or partial address describing the location of injury. Multiple lines are supported.</t>
+  </si>
+  <si>
+    <t>Certifier ID</t>
+  </si>
+  <si>
+    <t>Identifier of the Certifier such as NPI, SS, ID.
+Format: &lt;type&gt;:&lt;value&gt;
+Ex: NPI:1234567890</t>
   </si>
 </sst>
 </file>
@@ -1247,7 +1255,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1653,11 +1661,11 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
@@ -1749,16 +1757,8 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2093,18 +2093,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU76"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:AU77"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
     <col min="2" max="2" width="30.33203125" style="58" customWidth="1"/>
-    <col min="3" max="3" width="39.109375" style="65" customWidth="1"/>
-    <col min="4" max="8" width="32.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" style="65" customWidth="1"/>
+    <col min="4" max="8" width="32.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.77734375" style="1"/>
+    <col min="10" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
@@ -2133,12 +2133,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="23.4" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="65" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="105.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:9" ht="105.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="46" t="s">
         <v>9</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="4" customFormat="1" ht="34.799999999999997" thickTop="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:9" s="4" customFormat="1" ht="40" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47" t="s">
         <v>11</v>
       </c>
@@ -2162,7 +2162,7 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" s="6" customFormat="1" ht="29.4" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:9" s="6" customFormat="1" ht="31" x14ac:dyDescent="0.3">
       <c r="A5" s="48"/>
       <c r="B5" s="92" t="s">
         <v>13</v>
@@ -2177,7 +2177,7 @@
       <c r="H5" s="137"/>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" s="6" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:9" s="6" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A6" s="48"/>
       <c r="B6" s="93" t="s">
         <v>15</v>
@@ -2192,7 +2192,7 @@
       <c r="H6" s="137"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" s="8" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A7" s="49" t="s">
         <v>17</v>
       </c>
@@ -2207,7 +2207,7 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
     </row>
-    <row r="8" spans="1:9" s="11" customFormat="1" ht="68.400000000000006" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:9" s="11" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="50"/>
       <c r="B8" s="66" t="s">
         <v>19</v>
@@ -2222,7 +2222,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:9" s="11" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A9" s="50"/>
       <c r="B9" s="66" t="s">
         <v>21</v>
@@ -2237,7 +2237,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" s="11" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="50"/>
       <c r="B10" s="66" t="s">
         <v>24</v>
@@ -2252,7 +2252,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="10"/>
     </row>
-    <row r="11" spans="1:9" s="11" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:9" s="11" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A11" s="50"/>
       <c r="B11" s="67" t="s">
         <v>27</v>
@@ -2267,7 +2267,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:9" s="11" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A12" s="50"/>
       <c r="B12" s="66" t="s">
         <v>30</v>
@@ -2282,7 +2282,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:9" s="11" customFormat="1" ht="57" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:9" s="11" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A13" s="50"/>
       <c r="B13" s="66" t="s">
         <v>32</v>
@@ -2297,7 +2297,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9" s="11" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A14" s="50"/>
       <c r="B14" s="66" t="s">
         <v>34</v>
@@ -2312,7 +2312,7 @@
       <c r="H14" s="12"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="50"/>
       <c r="B15" s="66" t="s">
         <v>36</v>
@@ -2325,7 +2325,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" s="11" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A16" s="50"/>
       <c r="B16" s="66" t="s">
         <v>37</v>
@@ -2340,7 +2340,7 @@
       <c r="H16" s="9"/>
       <c r="I16" s="10"/>
     </row>
-    <row r="17" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="50"/>
       <c r="B17" s="66" t="s">
         <v>200</v>
@@ -2353,7 +2353,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="10"/>
     </row>
-    <row r="18" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="50"/>
       <c r="B18" s="66" t="s">
         <v>201</v>
@@ -2366,7 +2366,7 @@
       <c r="H18" s="9"/>
       <c r="I18" s="10"/>
     </row>
-    <row r="19" spans="1:9" s="11" customFormat="1" ht="26.4" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A19" s="50"/>
       <c r="B19" s="68" t="s">
         <v>39</v>
@@ -2379,7 +2379,7 @@
       <c r="H19" s="9"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="50"/>
       <c r="B20" s="66" t="s">
         <v>40</v>
@@ -2392,7 +2392,7 @@
       <c r="H20" s="9"/>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="50"/>
       <c r="B21" s="66" t="s">
         <v>41</v>
@@ -2405,7 +2405,7 @@
       <c r="H21" s="9"/>
       <c r="I21" s="10"/>
     </row>
-    <row r="22" spans="1:9" s="13" customFormat="1" ht="79.8" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:9" s="13" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A22" s="89" t="s">
         <v>42</v>
       </c>
@@ -2420,7 +2420,7 @@
       <c r="H22" s="139"/>
       <c r="I22" s="139"/>
     </row>
-    <row r="23" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="51"/>
       <c r="B23" s="94" t="s">
         <v>44</v>
@@ -2435,7 +2435,7 @@
       <c r="H23" s="14"/>
       <c r="I23" s="15"/>
     </row>
-    <row r="24" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="51"/>
       <c r="B24" s="94" t="s">
         <v>46</v>
@@ -2450,7 +2450,7 @@
       <c r="H24" s="17"/>
       <c r="I24" s="15"/>
     </row>
-    <row r="25" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="51"/>
       <c r="B25" s="94" t="s">
         <v>48</v>
@@ -2465,7 +2465,7 @@
       <c r="H25" s="18"/>
       <c r="I25" s="15"/>
     </row>
-    <row r="26" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="51"/>
       <c r="B26" s="94" t="s">
         <v>50</v>
@@ -2480,7 +2480,7 @@
       <c r="H26" s="18"/>
       <c r="I26" s="15"/>
     </row>
-    <row r="27" spans="1:9" s="16" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A27" s="51"/>
       <c r="B27" s="94" t="s">
         <v>52</v>
@@ -2495,7 +2495,7 @@
       <c r="H27" s="18"/>
       <c r="I27" s="15"/>
     </row>
-    <row r="28" spans="1:9" s="16" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A28" s="51"/>
       <c r="B28" s="94" t="s">
         <v>54</v>
@@ -2510,7 +2510,7 @@
       <c r="H28" s="18"/>
       <c r="I28" s="15"/>
     </row>
-    <row r="29" spans="1:9" s="16" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A29" s="51"/>
       <c r="B29" s="94" t="s">
         <v>56</v>
@@ -2525,7 +2525,7 @@
       <c r="H29" s="18"/>
       <c r="I29" s="15"/>
     </row>
-    <row r="30" spans="1:9" s="16" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A30" s="51"/>
       <c r="B30" s="94" t="s">
         <v>58</v>
@@ -2540,7 +2540,7 @@
       <c r="H30" s="14"/>
       <c r="I30" s="15"/>
     </row>
-    <row r="31" spans="1:9" s="16" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A31" s="51"/>
       <c r="B31" s="94" t="s">
         <v>60</v>
@@ -2555,7 +2555,7 @@
       <c r="H31" s="19"/>
       <c r="I31" s="15"/>
     </row>
-    <row r="32" spans="1:9" s="16" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:9" s="16" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A32" s="51"/>
       <c r="B32" s="69" t="s">
         <v>62</v>
@@ -2570,7 +2570,7 @@
       <c r="H32" s="19"/>
       <c r="I32" s="15"/>
     </row>
-    <row r="33" spans="1:9" s="16" customFormat="1" ht="57" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:9" s="16" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A33" s="51"/>
       <c r="B33" s="69" t="s">
         <v>65</v>
@@ -2585,7 +2585,7 @@
       <c r="H33" s="20"/>
       <c r="I33" s="15"/>
     </row>
-    <row r="34" spans="1:9" s="16" customFormat="1" ht="79.8" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:9" s="16" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A34" s="51"/>
       <c r="B34" s="69" t="s">
         <v>67</v>
@@ -2600,7 +2600,7 @@
       <c r="H34" s="21"/>
       <c r="I34" s="15"/>
     </row>
-    <row r="35" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="52"/>
       <c r="B35" s="69" t="s">
         <v>69</v>
@@ -2615,7 +2615,7 @@
       <c r="H35" s="18"/>
       <c r="I35" s="22"/>
     </row>
-    <row r="36" spans="1:9" s="16" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A36" s="51"/>
       <c r="B36" s="69" t="s">
         <v>71</v>
@@ -2630,7 +2630,7 @@
       <c r="H36" s="19"/>
       <c r="I36" s="15"/>
     </row>
-    <row r="37" spans="1:9" s="16" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A37" s="51"/>
       <c r="B37" s="69" t="s">
         <v>74</v>
@@ -2645,7 +2645,7 @@
       <c r="H37" s="19"/>
       <c r="I37" s="15"/>
     </row>
-    <row r="38" spans="1:9" s="25" customFormat="1" ht="79.8" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:9" s="25" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A38" s="90" t="s">
         <v>76</v>
       </c>
@@ -2660,7 +2660,7 @@
       <c r="H38" s="24"/>
       <c r="I38" s="24"/>
     </row>
-    <row r="39" spans="1:9" s="28" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A39" s="53"/>
       <c r="B39" s="70" t="s">
         <v>202</v>
@@ -2675,7 +2675,7 @@
       <c r="H39" s="26"/>
       <c r="I39" s="27"/>
     </row>
-    <row r="40" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="40" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="53"/>
       <c r="B40" s="70" t="s">
         <v>204</v>
@@ -2688,7 +2688,7 @@
       <c r="H40" s="26"/>
       <c r="I40" s="27"/>
     </row>
-    <row r="41" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="41" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="53"/>
       <c r="B41" s="70" t="s">
         <v>205</v>
@@ -2701,7 +2701,7 @@
       <c r="H41" s="26"/>
       <c r="I41" s="27"/>
     </row>
-    <row r="42" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="42" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="53"/>
       <c r="B42" s="70" t="s">
         <v>206</v>
@@ -2714,7 +2714,7 @@
       <c r="H42" s="26"/>
       <c r="I42" s="27"/>
     </row>
-    <row r="43" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="53"/>
       <c r="B43" s="70" t="s">
         <v>207</v>
@@ -2727,7 +2727,7 @@
       <c r="H43" s="26"/>
       <c r="I43" s="27"/>
     </row>
-    <row r="44" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="44" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="53"/>
       <c r="B44" s="70" t="s">
         <v>208</v>
@@ -2740,7 +2740,7 @@
       <c r="H44" s="26"/>
       <c r="I44" s="27"/>
     </row>
-    <row r="45" spans="1:9" s="28" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A45" s="53"/>
       <c r="B45" s="71" t="s">
         <v>209</v>
@@ -2748,79 +2748,79 @@
       <c r="C45" s="83" t="s">
         <v>215</v>
       </c>
-      <c r="D45" s="159"/>
-      <c r="E45" s="160"/>
-      <c r="F45" s="161"/>
-      <c r="G45" s="160"/>
-      <c r="H45" s="160"/>
+      <c r="D45" s="149"/>
+      <c r="E45" s="159"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="159"/>
+      <c r="H45" s="159"/>
       <c r="I45" s="27"/>
     </row>
-    <row r="46" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="46" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="53"/>
       <c r="B46" s="71" t="s">
         <v>210</v>
       </c>
       <c r="C46" s="83"/>
-      <c r="D46" s="159"/>
-      <c r="E46" s="160"/>
-      <c r="F46" s="161"/>
-      <c r="G46" s="160"/>
-      <c r="H46" s="160"/>
+      <c r="D46" s="149"/>
+      <c r="E46" s="159"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="159"/>
+      <c r="H46" s="159"/>
       <c r="I46" s="27"/>
     </row>
-    <row r="47" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="53"/>
       <c r="B47" s="71" t="s">
         <v>211</v>
       </c>
       <c r="C47" s="83"/>
-      <c r="D47" s="159"/>
-      <c r="E47" s="160"/>
-      <c r="F47" s="161"/>
-      <c r="G47" s="160"/>
-      <c r="H47" s="160"/>
+      <c r="D47" s="149"/>
+      <c r="E47" s="159"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="159"/>
+      <c r="H47" s="159"/>
       <c r="I47" s="27"/>
     </row>
-    <row r="48" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="53"/>
       <c r="B48" s="71" t="s">
         <v>212</v>
       </c>
       <c r="C48" s="83"/>
-      <c r="D48" s="159"/>
-      <c r="E48" s="160"/>
-      <c r="F48" s="161"/>
-      <c r="G48" s="160"/>
-      <c r="H48" s="160"/>
+      <c r="D48" s="149"/>
+      <c r="E48" s="159"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="159"/>
+      <c r="H48" s="159"/>
       <c r="I48" s="27"/>
     </row>
-    <row r="49" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="49" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="53"/>
       <c r="B49" s="71" t="s">
         <v>213</v>
       </c>
       <c r="C49" s="83"/>
-      <c r="D49" s="159"/>
-      <c r="E49" s="160"/>
-      <c r="F49" s="161"/>
-      <c r="G49" s="160"/>
-      <c r="H49" s="160"/>
+      <c r="D49" s="149"/>
+      <c r="E49" s="159"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="159"/>
+      <c r="H49" s="159"/>
       <c r="I49" s="27"/>
     </row>
-    <row r="50" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="50" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="53"/>
       <c r="B50" s="71" t="s">
         <v>214</v>
       </c>
       <c r="C50" s="83"/>
-      <c r="D50" s="159"/>
-      <c r="E50" s="160"/>
-      <c r="F50" s="161"/>
-      <c r="G50" s="160"/>
-      <c r="H50" s="160"/>
+      <c r="D50" s="149"/>
+      <c r="E50" s="159"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="159"/>
+      <c r="H50" s="159"/>
       <c r="I50" s="27"/>
     </row>
-    <row r="51" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="53"/>
       <c r="B51" s="70" t="s">
         <v>78</v>
@@ -2833,7 +2833,7 @@
       <c r="H51" s="149"/>
       <c r="I51" s="27"/>
     </row>
-    <row r="52" spans="1:47" s="28" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="52" spans="1:47" s="28" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A52" s="53"/>
       <c r="B52" s="91" t="s">
         <v>80</v>
@@ -2848,7 +2848,7 @@
       <c r="H52" s="26"/>
       <c r="I52" s="27"/>
     </row>
-    <row r="53" spans="1:47" s="31" customFormat="1" ht="57" x14ac:dyDescent="0.5">
+    <row r="53" spans="1:47" s="31" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A53" s="97" t="s">
         <v>82</v>
       </c>
@@ -2863,7 +2863,7 @@
       <c r="H53" s="29"/>
       <c r="I53" s="30"/>
     </row>
-    <row r="54" spans="1:47" s="34" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="54" spans="1:47" s="34" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A54" s="54"/>
       <c r="B54" s="72" t="s">
         <v>84</v>
@@ -2878,7 +2878,7 @@
       <c r="H54" s="32"/>
       <c r="I54" s="33"/>
     </row>
-    <row r="55" spans="1:47" s="34" customFormat="1" ht="79.8" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A55" s="54"/>
       <c r="B55" s="72" t="s">
         <v>86</v>
@@ -2893,7 +2893,7 @@
       <c r="H55" s="35"/>
       <c r="I55" s="33"/>
     </row>
-    <row r="56" spans="1:47" s="34" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="56" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A56" s="54"/>
       <c r="B56" s="72" t="s">
         <v>88</v>
@@ -2908,7 +2908,7 @@
       <c r="H56" s="148"/>
       <c r="I56" s="33"/>
     </row>
-    <row r="57" spans="1:47" s="34" customFormat="1" ht="57" x14ac:dyDescent="0.5">
+    <row r="57" spans="1:47" s="34" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A57" s="54"/>
       <c r="B57" s="72" t="s">
         <v>91</v>
@@ -2923,7 +2923,7 @@
       <c r="H57" s="36"/>
       <c r="I57" s="33"/>
     </row>
-    <row r="58" spans="1:47" s="34" customFormat="1" ht="91.2" x14ac:dyDescent="0.5">
+    <row r="58" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A58" s="54"/>
       <c r="B58" s="72" t="s">
         <v>93</v>
@@ -2938,7 +2938,7 @@
       <c r="H58" s="35"/>
       <c r="I58" s="33"/>
     </row>
-    <row r="59" spans="1:47" s="34" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="59" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A59" s="54"/>
       <c r="B59" s="72" t="s">
         <v>95</v>
@@ -2953,7 +2953,7 @@
       <c r="H59" s="148"/>
       <c r="I59" s="33"/>
     </row>
-    <row r="60" spans="1:47" s="38" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="60" spans="1:47" s="38" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A60" s="55" t="s">
         <v>98</v>
       </c>
@@ -2968,7 +2968,7 @@
       <c r="H60" s="37"/>
       <c r="I60" s="37"/>
     </row>
-    <row r="61" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="61" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="56"/>
       <c r="B61" s="73" t="s">
         <v>100</v>
@@ -2983,7 +2983,7 @@
       <c r="H61" s="39"/>
       <c r="I61" s="40"/>
     </row>
-    <row r="62" spans="1:47" s="41" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="62" spans="1:47" s="41" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A62" s="56"/>
       <c r="B62" s="73" t="s">
         <v>102</v>
@@ -2998,7 +2998,7 @@
       <c r="H62" s="39"/>
       <c r="I62" s="40"/>
     </row>
-    <row r="63" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="56"/>
       <c r="B63" s="73" t="s">
         <v>104</v>
@@ -3013,7 +3013,7 @@
       <c r="H63" s="155"/>
       <c r="I63" s="56"/>
     </row>
-    <row r="64" spans="1:47" s="42" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="64" spans="1:47" s="42" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A64" s="56"/>
       <c r="B64" s="73" t="s">
         <v>106</v>
@@ -3066,7 +3066,7 @@
       <c r="AT64" s="56"/>
       <c r="AU64" s="56"/>
     </row>
-    <row r="65" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="65" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="56"/>
       <c r="B65" s="73" t="s">
         <v>108</v>
@@ -3117,7 +3117,7 @@
       <c r="AT65" s="56"/>
       <c r="AU65" s="56"/>
     </row>
-    <row r="66" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="56"/>
       <c r="B66" s="73" t="s">
         <v>109</v>
@@ -3168,7 +3168,7 @@
       <c r="AT66" s="56"/>
       <c r="AU66" s="56"/>
     </row>
-    <row r="67" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="67" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="56"/>
       <c r="B67" s="73" t="s">
         <v>110</v>
@@ -3219,7 +3219,7 @@
       <c r="AT67" s="56"/>
       <c r="AU67" s="56"/>
     </row>
-    <row r="68" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="68" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="56"/>
       <c r="B68" s="73" t="s">
         <v>111</v>
@@ -3270,7 +3270,7 @@
       <c r="AT68" s="56"/>
       <c r="AU68" s="56"/>
     </row>
-    <row r="69" spans="1:47" s="105" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="69" spans="1:47" s="105" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="101" t="s">
         <v>165</v>
       </c>
@@ -3283,7 +3283,7 @@
       <c r="H69" s="104"/>
       <c r="I69" s="104"/>
     </row>
-    <row r="70" spans="1:47" s="45" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="70" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A70" s="57"/>
       <c r="B70" s="74" t="s">
         <v>112</v>
@@ -3298,7 +3298,7 @@
       <c r="H70" s="43"/>
       <c r="I70" s="44"/>
     </row>
-    <row r="71" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="71" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="57"/>
       <c r="B71" s="74" t="s">
         <v>114</v>
@@ -3311,7 +3311,7 @@
       <c r="H71" s="43"/>
       <c r="I71" s="44"/>
     </row>
-    <row r="72" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="72" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="57"/>
       <c r="B72" s="74" t="s">
         <v>115</v>
@@ -3324,7 +3324,7 @@
       <c r="H72" s="43"/>
       <c r="I72" s="44"/>
     </row>
-    <row r="73" spans="1:47" s="45" customFormat="1" ht="39.6" x14ac:dyDescent="0.5">
+    <row r="73" spans="1:47" s="45" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A73" s="57"/>
       <c r="B73" s="75" t="s">
         <v>116</v>
@@ -3337,7 +3337,7 @@
       <c r="H73" s="43"/>
       <c r="I73" s="44"/>
     </row>
-    <row r="74" spans="1:47" s="45" customFormat="1" ht="26.4" x14ac:dyDescent="0.5">
+    <row r="74" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A74" s="57"/>
       <c r="B74" s="75" t="s">
         <v>117</v>
@@ -3350,7 +3350,7 @@
       <c r="H74" s="43"/>
       <c r="I74" s="44"/>
     </row>
-    <row r="75" spans="1:47" s="45" customFormat="1" ht="68.400000000000006" x14ac:dyDescent="0.5">
+    <row r="75" spans="1:47" s="45" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A75" s="57"/>
       <c r="B75" s="74" t="s">
         <v>118</v>
@@ -3365,13 +3365,13 @@
       <c r="H75" s="43"/>
       <c r="I75" s="44"/>
     </row>
-    <row r="76" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="76" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A76" s="57"/>
       <c r="B76" s="74" t="s">
-        <v>120</v>
+        <v>216</v>
       </c>
       <c r="C76" s="88" t="s">
-        <v>121</v>
+        <v>217</v>
       </c>
       <c r="D76" s="156"/>
       <c r="E76" s="43"/>
@@ -3379,6 +3379,21 @@
       <c r="G76" s="43"/>
       <c r="H76" s="43"/>
       <c r="I76" s="44"/>
+    </row>
+    <row r="77" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="57"/>
+      <c r="B77" s="74" t="s">
+        <v>120</v>
+      </c>
+      <c r="C77" s="88" t="s">
+        <v>121</v>
+      </c>
+      <c r="D77" s="156"/>
+      <c r="E77" s="43"/>
+      <c r="F77" s="43"/>
+      <c r="G77" s="43"/>
+      <c r="H77" s="43"/>
+      <c r="I77" s="44"/>
     </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
@@ -3390,17 +3405,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C559A218-9020-4822-8346-393500FE199B}">
   <dimension ref="A1:I69"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
     <col min="2" max="2" width="30.33203125" style="58" customWidth="1"/>
-    <col min="3" max="3" width="39.109375" style="65" customWidth="1"/>
-    <col min="4" max="8" width="32.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" style="65" customWidth="1"/>
+    <col min="4" max="8" width="32.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.77734375" style="1"/>
+    <col min="10" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
@@ -3429,12 +3444,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="57" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:9" ht="65" x14ac:dyDescent="0.3">
       <c r="C2" s="65" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="114" customFormat="1" ht="34.200000000000003" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:9" s="114" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A3" s="112" t="s">
         <v>167</v>
       </c>
@@ -3449,7 +3464,7 @@
       <c r="H3" s="113"/>
       <c r="I3" s="113"/>
     </row>
-    <row r="4" spans="1:9" s="108" customFormat="1" ht="151.80000000000001" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:9" s="108" customFormat="1" ht="169" x14ac:dyDescent="0.3">
       <c r="A4" s="107"/>
       <c r="B4" s="109" t="s">
         <v>187</v>
@@ -3464,7 +3479,7 @@
       <c r="H4" s="111"/>
       <c r="I4" s="106"/>
     </row>
-    <row r="5" spans="1:9" s="108" customFormat="1" ht="68.400000000000006" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:9" s="108" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A5" s="107"/>
       <c r="B5" s="109" t="s">
         <v>168</v>
@@ -3479,7 +3494,7 @@
       <c r="H5" s="111"/>
       <c r="I5" s="106"/>
     </row>
-    <row r="6" spans="1:9" s="108" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A6" s="107"/>
       <c r="B6" s="109" t="s">
         <v>196</v>
@@ -3494,7 +3509,7 @@
       <c r="H6" s="111"/>
       <c r="I6" s="106"/>
     </row>
-    <row r="7" spans="1:9" s="108" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A7" s="107"/>
       <c r="B7" s="109" t="s">
         <v>195</v>
@@ -3509,7 +3524,7 @@
       <c r="H7" s="111"/>
       <c r="I7" s="106"/>
     </row>
-    <row r="8" spans="1:9" s="108" customFormat="1" ht="45.6" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:9" s="108" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A8" s="107"/>
       <c r="B8" s="109" t="s">
         <v>169</v>
@@ -3524,7 +3539,7 @@
       <c r="H8" s="111"/>
       <c r="I8" s="106"/>
     </row>
-    <row r="9" spans="1:9" s="129" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:9" s="129" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A9" s="125" t="s">
         <v>172</v>
       </c>
@@ -3539,7 +3554,7 @@
       <c r="H9" s="128"/>
       <c r="I9" s="128"/>
     </row>
-    <row r="10" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="117"/>
       <c r="B10" s="121" t="s">
         <v>173</v>
@@ -3554,7 +3569,7 @@
       <c r="H10" s="123"/>
       <c r="I10" s="119"/>
     </row>
-    <row r="11" spans="1:9" s="120" customFormat="1" ht="22.8" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:9" s="120" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A11" s="117"/>
       <c r="B11" s="121" t="s">
         <v>176</v>
@@ -3569,7 +3584,7 @@
       <c r="H11" s="123"/>
       <c r="I11" s="119"/>
     </row>
-    <row r="12" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="117"/>
       <c r="B12" s="121" t="s">
         <v>177</v>
@@ -3582,7 +3597,7 @@
       <c r="H12" s="123"/>
       <c r="I12" s="119"/>
     </row>
-    <row r="13" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="117"/>
       <c r="B13" s="121" t="s">
         <v>178</v>
@@ -3595,7 +3610,7 @@
       <c r="H13" s="123"/>
       <c r="I13" s="119"/>
     </row>
-    <row r="14" spans="1:9" s="120" customFormat="1" ht="39.6" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:9" s="120" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A14" s="117"/>
       <c r="B14" s="124" t="s">
         <v>179</v>
@@ -3608,7 +3623,7 @@
       <c r="H14" s="123"/>
       <c r="I14" s="119"/>
     </row>
-    <row r="15" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="117"/>
       <c r="B15" s="121" t="s">
         <v>180</v>
@@ -3621,7 +3636,7 @@
       <c r="H15" s="123"/>
       <c r="I15" s="119"/>
     </row>
-    <row r="16" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="117"/>
       <c r="B16" s="121" t="s">
         <v>181</v>
@@ -3634,7 +3649,7 @@
       <c r="H16" s="123"/>
       <c r="I16" s="119"/>
     </row>
-    <row r="17" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="117"/>
       <c r="B17" s="121" t="s">
         <v>183</v>
@@ -3649,7 +3664,7 @@
       <c r="H17" s="131"/>
       <c r="I17" s="119"/>
     </row>
-    <row r="18" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="117"/>
       <c r="B18" s="121" t="s">
         <v>184</v>
@@ -3664,57 +3679,57 @@
       <c r="H18" s="131"/>
       <c r="I18" s="119"/>
     </row>
-    <row r="19" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:9" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="33" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="34" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="35" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="36" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="37" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="38" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="39" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="40" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="41" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="42" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="43" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="44" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="45" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="46" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="47" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="48" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="49" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="50" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="51" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="52" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="53" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="54" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="56" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="57" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="58" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="60" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="61" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="62" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="63" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="64" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="65" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="66" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="67" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="69" customFormat="1" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="33" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="34" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="35" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="36" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="37" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="38" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="39" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="40" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="41" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="42" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="43" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="44" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="45" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="46" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="47" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="48" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="49" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="50" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="51" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="52" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="53" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="54" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="55" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="56" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="57" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="58" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="59" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="60" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="61" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="62" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="63" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="64" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="65" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="66" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="67" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="68" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="69" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -3754,25 +3769,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F8BFBD-18C1-4ED5-A02E-9841686C259E}">
   <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="32.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="62" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="49.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -3816,7 +3831,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -3860,7 +3875,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>137</v>
       </c>
@@ -3904,7 +3919,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>144</v>
       </c>
@@ -3948,7 +3963,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>155</v>
       </c>
@@ -3983,7 +3998,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -4006,7 +4021,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>145</v>
       </c>
@@ -4027,17 +4042,53 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
-      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
-      <Description>YVWEJ5DVYS2U-421999773-68</Description>
-    </_dlc_DocIdUrl>
-    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4240,53 +4291,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
+      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
+      <Description>YVWEJ5DVYS2U-421999773-68</Description>
+    </_dlc_DocIdUrl>
+    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4299,19 +4314,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4337,9 +4342,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
MDI and DCR import tested.
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF75D8B1-DCC4-0240-A3D0-DC3970BA3F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5B174C-5679-9249-A892-E06A50BC2EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Base Input Schema" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="232">
   <si>
     <t>Sections</t>
   </si>
@@ -498,9 +498,6 @@
     <t>Is the Certifer a Physician, a pronouncer, or other?</t>
   </si>
   <si>
-    <t>Medical Examiner/Coroner</t>
-  </si>
-  <si>
     <t>Decedent Gender</t>
   </si>
   <si>
@@ -561,9 +558,6 @@
     <t>Pregnant at time of death</t>
   </si>
   <si>
-    <t>Pronouncing &amp; Certifying physician</t>
-  </si>
-  <si>
     <t>Black or African American</t>
   </si>
   <si>
@@ -592,9 +586,6 @@
   </si>
   <si>
     <t>Not pregnant, but pregnant within 42 days of death</t>
-  </si>
-  <si>
-    <t>Certifying Physician</t>
   </si>
   <si>
     <t>Native Hawaiian or Other Pacific Islander</t>
@@ -911,9 +902,61 @@
     <t>Certifier ID</t>
   </si>
   <si>
-    <t>Identifier of the Certifier such as NPI, SS, ID.
-Format: &lt;type&gt;:&lt;value&gt;
-Ex: NPI:1234567890</t>
+    <t>Certified Date</t>
+  </si>
+  <si>
+    <t>Date of Certification</t>
+  </si>
+  <si>
+    <t>Certifier ID System</t>
+  </si>
+  <si>
+    <t>Identifier System of the Certifier such as NPI, SS, ID.
+Ex: NPI</t>
+  </si>
+  <si>
+    <t>Identifier Value of the Certifier 
+Format is based on the ID system
+Ex: 1234567890</t>
+  </si>
+  <si>
+    <t>Death certification by medical examiner or coroner (procedure)</t>
+  </si>
+  <si>
+    <t>Death certification and verification by physician (procedure)</t>
+  </si>
+  <si>
+    <t>Death certification by physician (procedure)</t>
+  </si>
+  <si>
+    <t>Cremation Clearance Info</t>
+  </si>
+  <si>
+    <t>Funeral Home: Name</t>
+  </si>
+  <si>
+    <t>Funeral Home: Street</t>
+  </si>
+  <si>
+    <t>Funeral Home: City</t>
+  </si>
+  <si>
+    <t>Funeral Home: County</t>
+  </si>
+  <si>
+    <t>Funeral Home: State, U.S. Territory or Canadian Province</t>
+  </si>
+  <si>
+    <t>Funeral Home: Postal Code</t>
+  </si>
+  <si>
+    <t>Funeral Business Name</t>
+  </si>
+  <si>
+    <t>Funeral Home: Phone</t>
+  </si>
+  <si>
+    <t>Funeral Home: Fax</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1055,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="24">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1148,6 +1191,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDBD7FD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8470FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border>
@@ -1255,7 +1310,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1759,6 +1814,37 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1773,6 +1859,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF8470FF"/>
+      <color rgb="FFDBD7FD"/>
+      <color rgb="FFC1ABFF"/>
       <color rgb="FF637A3A"/>
       <color rgb="FF4D5F2D"/>
       <color rgb="FF9FBA6E"/>
@@ -1780,9 +1869,6 @@
       <color rgb="FF88723C"/>
       <color rgb="FFFFC32D"/>
       <color rgb="FFF48484"/>
-      <color rgb="FFC9C9C9"/>
-      <color rgb="FFF5D5A1"/>
-      <color rgb="FFF1C67F"/>
     </mruColors>
   </colors>
   <extLst>
@@ -2093,7 +2179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU77"/>
+  <dimension ref="A1:AU88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
@@ -2135,7 +2221,7 @@
     </row>
     <row r="2" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="65" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="105.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2343,7 +2429,7 @@
     <row r="17" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="50"/>
       <c r="B17" s="66" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C17" s="79"/>
       <c r="D17" s="138"/>
@@ -2356,7 +2442,7 @@
     <row r="18" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="50"/>
       <c r="B18" s="66" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C18" s="79"/>
       <c r="D18" s="138"/>
@@ -2663,10 +2749,10 @@
     <row r="39" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A39" s="53"/>
       <c r="B39" s="70" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C39" s="83" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D39" s="149"/>
       <c r="E39" s="26"/>
@@ -2678,7 +2764,7 @@
     <row r="40" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="53"/>
       <c r="B40" s="70" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C40" s="83"/>
       <c r="D40" s="149"/>
@@ -2691,7 +2777,7 @@
     <row r="41" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="53"/>
       <c r="B41" s="70" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C41" s="83"/>
       <c r="D41" s="149"/>
@@ -2704,7 +2790,7 @@
     <row r="42" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="53"/>
       <c r="B42" s="70" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C42" s="83"/>
       <c r="D42" s="149"/>
@@ -2717,7 +2803,7 @@
     <row r="43" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="53"/>
       <c r="B43" s="70" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C43" s="83"/>
       <c r="D43" s="149"/>
@@ -2730,7 +2816,7 @@
     <row r="44" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="53"/>
       <c r="B44" s="70" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C44" s="83"/>
       <c r="D44" s="149"/>
@@ -2743,10 +2829,10 @@
     <row r="45" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A45" s="53"/>
       <c r="B45" s="71" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C45" s="83" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D45" s="149"/>
       <c r="E45" s="159"/>
@@ -2758,7 +2844,7 @@
     <row r="46" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="53"/>
       <c r="B46" s="71" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C46" s="83"/>
       <c r="D46" s="149"/>
@@ -2771,7 +2857,7 @@
     <row r="47" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="53"/>
       <c r="B47" s="71" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C47" s="83"/>
       <c r="D47" s="149"/>
@@ -2784,7 +2870,7 @@
     <row r="48" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="53"/>
       <c r="B48" s="71" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C48" s="83"/>
       <c r="D48" s="149"/>
@@ -2797,7 +2883,7 @@
     <row r="49" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="53"/>
       <c r="B49" s="71" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C49" s="83"/>
       <c r="D49" s="149"/>
@@ -2810,7 +2896,7 @@
     <row r="50" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="53"/>
       <c r="B50" s="71" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C50" s="83"/>
       <c r="D50" s="149"/>
@@ -3272,7 +3358,7 @@
     </row>
     <row r="69" spans="1:47" s="105" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="101" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B69" s="102"/>
       <c r="C69" s="103"/>
@@ -3324,7 +3410,7 @@
       <c r="H72" s="43"/>
       <c r="I72" s="44"/>
     </row>
-    <row r="73" spans="1:47" s="45" customFormat="1" ht="42" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A73" s="57"/>
       <c r="B73" s="75" t="s">
         <v>116</v>
@@ -3365,7 +3451,7 @@
       <c r="H75" s="43"/>
       <c r="I75" s="44"/>
     </row>
-    <row r="76" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A76" s="57"/>
       <c r="B76" s="74" t="s">
         <v>216</v>
@@ -3380,13 +3466,13 @@
       <c r="H76" s="43"/>
       <c r="I76" s="44"/>
     </row>
-    <row r="77" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A77" s="57"/>
       <c r="B77" s="74" t="s">
-        <v>120</v>
+        <v>213</v>
       </c>
       <c r="C77" s="88" t="s">
-        <v>121</v>
+        <v>218</v>
       </c>
       <c r="D77" s="156"/>
       <c r="E77" s="43"/>
@@ -3395,10 +3481,171 @@
       <c r="H77" s="43"/>
       <c r="I77" s="44"/>
     </row>
+    <row r="78" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="57"/>
+      <c r="B78" s="74" t="s">
+        <v>214</v>
+      </c>
+      <c r="C78" s="88" t="s">
+        <v>215</v>
+      </c>
+      <c r="D78" s="156"/>
+      <c r="E78" s="43"/>
+      <c r="F78" s="43"/>
+      <c r="G78" s="43"/>
+      <c r="H78" s="43"/>
+      <c r="I78" s="44"/>
+    </row>
+    <row r="79" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="57"/>
+      <c r="B79" s="74" t="s">
+        <v>120</v>
+      </c>
+      <c r="C79" s="88" t="s">
+        <v>121</v>
+      </c>
+      <c r="D79" s="156"/>
+      <c r="E79" s="43"/>
+      <c r="F79" s="43"/>
+      <c r="G79" s="43"/>
+      <c r="H79" s="43"/>
+      <c r="I79" s="44"/>
+    </row>
+    <row r="80" spans="1:47" s="167" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="163" t="s">
+        <v>222</v>
+      </c>
+      <c r="B80" s="164"/>
+      <c r="C80" s="165"/>
+      <c r="D80" s="166"/>
+      <c r="E80" s="166"/>
+      <c r="F80" s="166"/>
+      <c r="G80" s="166"/>
+      <c r="H80" s="166"/>
+      <c r="I80" s="166"/>
+    </row>
+    <row r="81" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="160"/>
+      <c r="B81" s="168" t="s">
+        <v>223</v>
+      </c>
+      <c r="C81" s="169" t="s">
+        <v>229</v>
+      </c>
+      <c r="D81" s="170"/>
+      <c r="E81" s="170"/>
+      <c r="F81" s="170"/>
+      <c r="G81" s="170"/>
+      <c r="H81" s="170"/>
+      <c r="I81" s="161"/>
+    </row>
+    <row r="82" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="160"/>
+      <c r="B82" s="168" t="s">
+        <v>230</v>
+      </c>
+      <c r="C82" s="169"/>
+      <c r="D82" s="170"/>
+      <c r="E82" s="170"/>
+      <c r="F82" s="170"/>
+      <c r="G82" s="170"/>
+      <c r="H82" s="170"/>
+      <c r="I82" s="161"/>
+    </row>
+    <row r="83" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="160"/>
+      <c r="B83" s="168" t="s">
+        <v>231</v>
+      </c>
+      <c r="C83" s="169"/>
+      <c r="D83" s="170"/>
+      <c r="E83" s="170"/>
+      <c r="F83" s="170"/>
+      <c r="G83" s="170"/>
+      <c r="H83" s="170"/>
+      <c r="I83" s="161"/>
+    </row>
+    <row r="84" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="160"/>
+      <c r="B84" s="168" t="s">
+        <v>224</v>
+      </c>
+      <c r="C84" s="169"/>
+      <c r="D84" s="170"/>
+      <c r="E84" s="170"/>
+      <c r="F84" s="170"/>
+      <c r="G84" s="170"/>
+      <c r="H84" s="170"/>
+      <c r="I84" s="161"/>
+    </row>
+    <row r="85" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="160"/>
+      <c r="B85" s="168" t="s">
+        <v>225</v>
+      </c>
+      <c r="C85" s="169"/>
+      <c r="D85" s="170"/>
+      <c r="E85" s="170"/>
+      <c r="F85" s="170"/>
+      <c r="G85" s="170"/>
+      <c r="H85" s="170"/>
+      <c r="I85" s="161"/>
+    </row>
+    <row r="86" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="160"/>
+      <c r="B86" s="168" t="s">
+        <v>226</v>
+      </c>
+      <c r="C86" s="169"/>
+      <c r="D86" s="170"/>
+      <c r="E86" s="170"/>
+      <c r="F86" s="170"/>
+      <c r="G86" s="170"/>
+      <c r="H86" s="170"/>
+      <c r="I86" s="161"/>
+    </row>
+    <row r="87" spans="1:9" s="162" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A87" s="160"/>
+      <c r="B87" s="171" t="s">
+        <v>227</v>
+      </c>
+      <c r="C87" s="169"/>
+      <c r="D87" s="170"/>
+      <c r="E87" s="170"/>
+      <c r="F87" s="170"/>
+      <c r="G87" s="170"/>
+      <c r="H87" s="170"/>
+      <c r="I87" s="161"/>
+    </row>
+    <row r="88" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="160"/>
+      <c r="B88" s="168" t="s">
+        <v>228</v>
+      </c>
+      <c r="C88" s="169"/>
+      <c r="D88" s="170"/>
+      <c r="E88" s="170"/>
+      <c r="F88" s="170"/>
+      <c r="G88" s="170"/>
+      <c r="H88" s="170"/>
+      <c r="I88" s="161"/>
+    </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{50949F61-4BF7-AF4C-825F-13906CC8DAFA}">
+          <x14:formula1>
+            <xm:f>'Drop Down List Values'!$M$2:$M$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>D79:H79</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -3446,12 +3693,12 @@
     </row>
     <row r="2" spans="1:9" ht="65" x14ac:dyDescent="0.3">
       <c r="C2" s="65" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="114" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A3" s="112" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B3" s="115"/>
       <c r="C3" s="116" t="s">
@@ -3467,10 +3714,10 @@
     <row r="4" spans="1:9" s="108" customFormat="1" ht="169" x14ac:dyDescent="0.3">
       <c r="A4" s="107"/>
       <c r="B4" s="109" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C4" s="110" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D4" s="111"/>
       <c r="E4" s="111"/>
@@ -3482,10 +3729,10 @@
     <row r="5" spans="1:9" s="108" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A5" s="107"/>
       <c r="B5" s="109" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C5" s="110" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D5" s="111"/>
       <c r="E5" s="111"/>
@@ -3497,10 +3744,10 @@
     <row r="6" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A6" s="107"/>
       <c r="B6" s="109" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C6" s="110" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D6" s="111"/>
       <c r="E6" s="111"/>
@@ -3512,10 +3759,10 @@
     <row r="7" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A7" s="107"/>
       <c r="B7" s="109" t="s">
+        <v>192</v>
+      </c>
+      <c r="C7" s="110" t="s">
         <v>195</v>
-      </c>
-      <c r="C7" s="110" t="s">
-        <v>198</v>
       </c>
       <c r="D7" s="111"/>
       <c r="E7" s="111"/>
@@ -3527,10 +3774,10 @@
     <row r="8" spans="1:9" s="108" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A8" s="107"/>
       <c r="B8" s="109" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C8" s="110" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D8" s="134"/>
       <c r="E8" s="111"/>
@@ -3541,11 +3788,11 @@
     </row>
     <row r="9" spans="1:9" s="129" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A9" s="125" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B9" s="126"/>
       <c r="C9" s="127" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D9" s="128"/>
       <c r="E9" s="128"/>
@@ -3557,10 +3804,10 @@
     <row r="10" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="117"/>
       <c r="B10" s="121" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C10" s="118" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D10" s="122"/>
       <c r="E10" s="123"/>
@@ -3572,10 +3819,10 @@
     <row r="11" spans="1:9" s="120" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A11" s="117"/>
       <c r="B11" s="121" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C11" s="118" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D11" s="135"/>
       <c r="E11" s="136"/>
@@ -3587,7 +3834,7 @@
     <row r="12" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="117"/>
       <c r="B12" s="121" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C12" s="118"/>
       <c r="D12" s="122"/>
@@ -3600,7 +3847,7 @@
     <row r="13" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="117"/>
       <c r="B13" s="121" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C13" s="118"/>
       <c r="D13" s="122"/>
@@ -3613,7 +3860,7 @@
     <row r="14" spans="1:9" s="120" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A14" s="117"/>
       <c r="B14" s="124" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C14" s="118"/>
       <c r="D14" s="122"/>
@@ -3626,7 +3873,7 @@
     <row r="15" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="117"/>
       <c r="B15" s="121" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C15" s="118"/>
       <c r="D15" s="122"/>
@@ -3639,7 +3886,7 @@
     <row r="16" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="117"/>
       <c r="B16" s="121" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C16" s="118"/>
       <c r="D16" s="122"/>
@@ -3652,10 +3899,10 @@
     <row r="17" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="117"/>
       <c r="B17" s="121" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C17" s="118" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D17" s="130"/>
       <c r="E17" s="131"/>
@@ -3667,10 +3914,10 @@
     <row r="18" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="117"/>
       <c r="B18" s="121" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C18" s="118" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D18" s="132"/>
       <c r="E18" s="133"/>
@@ -3795,48 +4042,48 @@
         <v>24</v>
       </c>
       <c r="C1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" t="s">
         <v>123</v>
-      </c>
-      <c r="D1" t="s">
-        <v>124</v>
       </c>
       <c r="E1" t="s">
         <v>62</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G1" t="s">
         <v>74</v>
       </c>
       <c r="H1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I1" t="s">
         <v>80</v>
       </c>
       <c r="J1" t="s">
+        <v>126</v>
+      </c>
+      <c r="K1" t="s">
         <v>127</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>128</v>
-      </c>
-      <c r="L1" t="s">
-        <v>129</v>
       </c>
       <c r="M1" t="s">
         <v>120</v>
       </c>
       <c r="N1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" t="s">
         <v>130</v>
-      </c>
-      <c r="B2" t="s">
-        <v>131</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
@@ -3845,48 +4092,48 @@
         <v>29</v>
       </c>
       <c r="E2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F2" t="s">
         <v>132</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>133</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I2" t="s">
+        <v>132</v>
+      </c>
+      <c r="J2" t="s">
         <v>134</v>
-      </c>
-      <c r="H2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I2" t="s">
-        <v>133</v>
-      </c>
-      <c r="J2" t="s">
-        <v>135</v>
       </c>
       <c r="K2" t="s">
         <v>90</v>
       </c>
       <c r="L2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M2" t="s">
-        <v>122</v>
+        <v>219</v>
       </c>
       <c r="N2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E3" t="s">
         <v>64</v>
@@ -3895,7 +4142,7 @@
         <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H3" t="s">
         <v>73</v>
@@ -3904,80 +4151,80 @@
         <v>73</v>
       </c>
       <c r="J3" t="s">
+        <v>139</v>
+      </c>
+      <c r="K3" t="s">
         <v>140</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>141</v>
       </c>
-      <c r="L3" t="s">
-        <v>142</v>
-      </c>
       <c r="M3" t="s">
-        <v>143</v>
+        <v>220</v>
       </c>
       <c r="N3" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" t="s">
         <v>144</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>145</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>146</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" t="s">
         <v>147</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H4" t="s">
+        <v>143</v>
+      </c>
+      <c r="I4" t="s">
         <v>148</v>
       </c>
-      <c r="F4" t="s">
-        <v>145</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="J4" t="s">
         <v>149</v>
       </c>
-      <c r="H4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>150</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>151</v>
       </c>
-      <c r="K4" t="s">
-        <v>152</v>
-      </c>
-      <c r="L4" t="s">
-        <v>153</v>
-      </c>
       <c r="M4" t="s">
-        <v>154</v>
+        <v>221</v>
       </c>
       <c r="N4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F5" t="s">
         <v>79</v>
@@ -3986,16 +4233,19 @@
         <v>79</v>
       </c>
       <c r="I5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J5" t="s">
         <v>97</v>
       </c>
       <c r="L5" t="s">
-        <v>158</v>
+        <v>155</v>
+      </c>
+      <c r="M5" t="s">
+        <v>144</v>
       </c>
       <c r="N5" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -4003,33 +4253,33 @@
         <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E6" t="s">
+        <v>156</v>
+      </c>
+      <c r="I6" t="s">
+        <v>157</v>
+      </c>
+      <c r="J6" t="s">
+        <v>158</v>
+      </c>
+      <c r="L6" t="s">
         <v>159</v>
       </c>
-      <c r="I6" t="s">
-        <v>160</v>
-      </c>
-      <c r="J6" t="s">
-        <v>161</v>
-      </c>
-      <c r="L6" t="s">
-        <v>162</v>
-      </c>
       <c r="N6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="L7" t="s">
         <v>79</v>
@@ -4092,6 +4342,29 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
+      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
+      <Description>YVWEJ5DVYS2U-421999773-68</Description>
+    </_dlc_DocIdUrl>
+    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D4902BA52C7D94A994657A564808B2B" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4455a60d2ff5f5fcd8815d6d89b5b66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b541edd5-2552-480e-ada6-0e2c8d317108" xmlns:ns3="780ae317-08c5-4e10-af93-dd385a8384a9" xmlns:ns4="3146657c-56f4-4c0a-bb9c-a675121ac670" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1d01ecd782f081d5d944fa263943fc4" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="b541edd5-2552-480e-ada6-0e2c8d317108"/>
@@ -4290,29 +4563,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
-      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
-      <Description>YVWEJ5DVYS2U-421999773-68</Description>
-    </_dlc_DocIdUrl>
-    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
   <ds:schemaRefs>
@@ -4322,21 +4572,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
-    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
-    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4360,9 +4598,21 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
+    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
+    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Funeral home director added
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A1659C-6787-5D43-B12E-4FC4BCD5063B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D7E804-6C0A-8C43-8919-0C8F579A1437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="840" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="236">
   <si>
     <t>Sections</t>
   </si>
@@ -963,6 +963,12 @@
   </si>
   <si>
     <t>Signature in image</t>
+  </si>
+  <si>
+    <t>Funeral Home: Director Name</t>
+  </si>
+  <si>
+    <t>Funeral Home Director (or Authorized) Name who is authoritative person for the DCR request</t>
   </si>
 </sst>
 </file>
@@ -2196,7 +2202,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU89"/>
+  <dimension ref="A1:AU90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
@@ -3556,12 +3562,14 @@
       <c r="H81" s="170"/>
       <c r="I81" s="161"/>
     </row>
-    <row r="82" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" s="162" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A82" s="160"/>
       <c r="B82" s="168" t="s">
-        <v>230</v>
-      </c>
-      <c r="C82" s="169"/>
+        <v>234</v>
+      </c>
+      <c r="C82" s="169" t="s">
+        <v>235</v>
+      </c>
       <c r="D82" s="170"/>
       <c r="E82" s="170"/>
       <c r="F82" s="170"/>
@@ -3572,7 +3580,7 @@
     <row r="83" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="160"/>
       <c r="B83" s="168" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C83" s="169"/>
       <c r="D83" s="170"/>
@@ -3585,7 +3593,7 @@
     <row r="84" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A84" s="160"/>
       <c r="B84" s="168" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C84" s="169"/>
       <c r="D84" s="170"/>
@@ -3598,7 +3606,7 @@
     <row r="85" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="160"/>
       <c r="B85" s="168" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C85" s="169"/>
       <c r="D85" s="170"/>
@@ -3611,7 +3619,7 @@
     <row r="86" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="160"/>
       <c r="B86" s="168" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C86" s="169"/>
       <c r="D86" s="170"/>
@@ -3621,10 +3629,10 @@
       <c r="H86" s="170"/>
       <c r="I86" s="161"/>
     </row>
-    <row r="87" spans="1:9" s="162" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="160"/>
-      <c r="B87" s="171" t="s">
-        <v>227</v>
+      <c r="B87" s="168" t="s">
+        <v>226</v>
       </c>
       <c r="C87" s="169"/>
       <c r="D87" s="170"/>
@@ -3634,10 +3642,10 @@
       <c r="H87" s="170"/>
       <c r="I87" s="161"/>
     </row>
-    <row r="88" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" s="162" customFormat="1" ht="31" x14ac:dyDescent="0.3">
       <c r="A88" s="160"/>
-      <c r="B88" s="168" t="s">
-        <v>228</v>
+      <c r="B88" s="171" t="s">
+        <v>227</v>
       </c>
       <c r="C88" s="169"/>
       <c r="D88" s="170"/>
@@ -3649,18 +3657,31 @@
     </row>
     <row r="89" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="160"/>
-      <c r="B89" s="172" t="s">
-        <v>232</v>
-      </c>
-      <c r="C89" s="169" t="s">
-        <v>233</v>
-      </c>
+      <c r="B89" s="168" t="s">
+        <v>228</v>
+      </c>
+      <c r="C89" s="169"/>
       <c r="D89" s="170"/>
       <c r="E89" s="170"/>
       <c r="F89" s="170"/>
       <c r="G89" s="170"/>
       <c r="H89" s="170"/>
       <c r="I89" s="161"/>
+    </row>
+    <row r="90" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="160"/>
+      <c r="B90" s="172" t="s">
+        <v>232</v>
+      </c>
+      <c r="C90" s="169" t="s">
+        <v>233</v>
+      </c>
+      <c r="D90" s="170"/>
+      <c r="E90" s="170"/>
+      <c r="F90" s="170"/>
+      <c r="G90" s="170"/>
+      <c r="H90" s="170"/>
+      <c r="I90" s="161"/>
     </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
@@ -4324,6 +4345,79 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
+      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
+      <Description>YVWEJ5DVYS2U-421999773-68</Description>
+    </_dlc_DocIdUrl>
+    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D4902BA52C7D94A994657A564808B2B" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4455a60d2ff5f5fcd8815d6d89b5b66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b541edd5-2552-480e-ada6-0e2c8d317108" xmlns:ns3="780ae317-08c5-4e10-af93-dd385a8384a9" xmlns:ns4="3146657c-56f4-4c0a-bb9c-a675121ac670" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1d01ecd782f081d5d944fa263943fc4" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="b541edd5-2552-480e-ada6-0e2c8d317108"/>
@@ -4522,80 +4616,41 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
-      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
-      <Description>YVWEJ5DVYS2U-421999773-68</Description>
-    </_dlc_DocIdUrl>
-    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4613,38 +4668,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated xlsx template and fix DCR CCR code
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D7E804-6C0A-8C43-8919-0C8F579A1437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F18E4E-07B4-5244-BD00-89625AC1620F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="840" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Base Input Schema" sheetId="4" r:id="rId1"/>
-    <sheet name="DCR Extension Input Schema" sheetId="6" r:id="rId2"/>
-    <sheet name="Drop Down List Values" sheetId="5" r:id="rId3"/>
+    <sheet name="DCR" sheetId="4" r:id="rId1"/>
+    <sheet name="Drop Down List Values" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="215">
   <si>
     <t>Sections</t>
   </si>
@@ -621,203 +620,6 @@
     <t>Medical Examiner</t>
   </si>
   <si>
-    <t>This Excel File can be imported into RAVEN2.0; converting into FHIR and importing into RAVEN. This tab describes the DCR specific data need for a Death Certificate Review, extending upon the "Base Input Schema"</t>
-  </si>
-  <si>
-    <t>Message Info</t>
-  </si>
-  <si>
-    <t>Submittor Name</t>
-  </si>
-  <si>
-    <t>Submittor Email</t>
-  </si>
-  <si>
-    <t>Name of the person who is submitting the Death Certificate Review Message
-Accepted Formats:
-&lt;First Name&gt; &lt;Last Name&gt;
-&lt;First Name&gt; &lt;Middle Initial&gt; &lt;Last Name&gt;
-&lt;First Name&gt; &lt;Middle Name&gt; &lt;Last Name&gt;</t>
-  </si>
-  <si>
-    <t>Email Addres of the person who is submitting the Death Certificate Review Message
-Accepted Formats:
-&lt;address&gt;@&lt;domain&gt;</t>
-  </si>
-  <si>
-    <t>Funeral Home</t>
-  </si>
-  <si>
-    <t>Funeral Home Name</t>
-  </si>
-  <si>
-    <t>This section is for The Funeral Home which admitted the body</t>
-  </si>
-  <si>
-    <t>Name of the admitting funeral home</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: Street</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: city</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: county</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: State, U.S. Territory or Canadian Province</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: Postal Code</t>
-  </si>
-  <si>
-    <t>Funeral Home Address: Country</t>
-  </si>
-  <si>
-    <t>Primary address of the funeral home. Multiple lines are supported</t>
-  </si>
-  <si>
-    <t>Funeral Home Phone Number</t>
-  </si>
-  <si>
-    <t>Funeral Home Fax Number</t>
-  </si>
-  <si>
-    <t>Primary Contact Phone Number of Funeral Home</t>
-  </si>
-  <si>
-    <t>Primary Fax Address of Funeral Home</t>
-  </si>
-  <si>
-    <t>Message Reason</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Context for why this message is being sent. Accepted Values shown in the dropdown
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>DC_MED_DATA_Q_REQ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Death Certificate Medical Data Quality Review Request
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>DC_MED_DATA_Q_RSP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Death Certificate Medical Data Quality Review Response
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>DC_PER_DATA_Q_REQ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Death Certificate Personal Data Quality Review Request
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>DC_PER_DATA_Q_RSP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Death Certificate Personal Data Quality Review Response
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>CREM_C_REQ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Cremation Clearance Request
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>CREM_C_RSP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">	  Cremation Clearance Response</t>
-    </r>
-  </si>
-  <si>
     <t>DC_MED_DATA_Q_REQ</t>
   </si>
   <si>
@@ -834,21 +636,6 @@
   </si>
   <si>
     <t>CREM_C_RSP</t>
-  </si>
-  <si>
-    <t>Submittor Fax Number</t>
-  </si>
-  <si>
-    <t>Submittor Phone Number</t>
-  </si>
-  <si>
-    <t>Primary Contact Phone Number of the person who is submitting the Death Certificate Review Message</t>
-  </si>
-  <si>
-    <t>Primary Fax Address of the person who is submitting the Death Certificate Review Message</t>
-  </si>
-  <si>
-    <t>This Excel File can be imported into RAVEN2.0; converting into FHIR and importing into RAVEN</t>
   </si>
   <si>
     <t>Decedent Residence: City</t>
@@ -969,17 +756,37 @@
   </si>
   <si>
     <t>Funeral Home Director (or Authorized) Name who is authoritative person for the DCR request</t>
+  </si>
+  <si>
+    <t>This Excel File can be imported into RAVEN. Mapping data in this file to Death Certificate Review (DCR) FHIR Profile</t>
+  </si>
+  <si>
+    <t>Usecase</t>
+  </si>
+  <si>
+    <t>Death Certificate Review (DCR) FHIR Profile</t>
+  </si>
+  <si>
+    <t>Funeral Home: Director ID System</t>
+  </si>
+  <si>
+    <t>Funeral Home: Director ID</t>
+  </si>
+  <si>
+    <t>Funeral Home Director's identifier system</t>
+  </si>
+  <si>
+    <t>Funeral Home Director's identifier value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-    <numFmt numFmtId="165" formatCode="[&lt;=9999999]###\-####;\(###\)\ ###\-####"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1052,21 +859,6 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -1075,7 +867,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1184,30 +976,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC48C00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF88723C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9FBA6E"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF637A3A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1322,15 +1090,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1511,47 +1278,15 @@
     <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1613,9 +1348,6 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1635,9 +1367,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1648,232 +1377,180 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="14" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="20" borderId="1" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="14" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="5">
     <cellStyle name="Bad" xfId="4" builtinId="27"/>
     <cellStyle name="Good" xfId="3" builtinId="26"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{40ABF838-51BB-482E-A30F-1A2350126FD1}"/>
@@ -2202,12 +1879,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU90"/>
+  <dimension ref="A1:AU92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" style="58" customWidth="1"/>
-    <col min="3" max="3" width="39.1640625" style="65" customWidth="1"/>
+    <col min="2" max="2" width="24.5" style="123" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" style="58" customWidth="1"/>
     <col min="4" max="8" width="32.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="8.83203125" style="1"/>
@@ -2217,10 +1894,10 @@
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="123" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="58" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -2242,17 +1919,23 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="65" t="s">
-        <v>196</v>
+    <row r="2" spans="1:9" ht="40" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="46" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="123" t="s">
+        <v>210</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="105.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="96" t="s">
+      <c r="B3" s="124"/>
+      <c r="C3" s="81" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2260,8 +1943,8 @@
       <c r="A4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="76" t="s">
+      <c r="B4" s="125"/>
+      <c r="C4" s="62" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="3"/>
@@ -2273,40 +1956,40 @@
     </row>
     <row r="5" spans="1:9" s="6" customFormat="1" ht="31" x14ac:dyDescent="0.3">
       <c r="A5" s="48"/>
-      <c r="B5" s="92" t="s">
+      <c r="B5" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="77" t="s">
+      <c r="C5" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
-      <c r="H5" s="137"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
       <c r="I5" s="5"/>
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A6" s="48"/>
-      <c r="B6" s="93" t="s">
+      <c r="B6" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="C6" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="137"/>
-      <c r="E6" s="137"/>
-      <c r="F6" s="137"/>
-      <c r="G6" s="137"/>
-      <c r="H6" s="137"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
       <c r="I6" s="5"/>
     </row>
     <row r="7" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A7" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="60"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="126"/>
+      <c r="C7" s="64" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="7"/>
@@ -2318,13 +2001,13 @@
     </row>
     <row r="8" spans="1:9" s="11" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="50"/>
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="79" t="s">
+      <c r="C8" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="138"/>
+      <c r="D8" s="91"/>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
@@ -2333,13 +2016,13 @@
     </row>
     <row r="9" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A9" s="50"/>
-      <c r="B9" s="66" t="s">
+      <c r="B9" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="79" t="s">
+      <c r="C9" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="138"/>
+      <c r="D9" s="91"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
@@ -2348,13 +2031,13 @@
     </row>
     <row r="10" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="50"/>
-      <c r="B10" s="66" t="s">
+      <c r="B10" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="79" t="s">
+      <c r="C10" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="138"/>
+      <c r="D10" s="91"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -2363,13 +2046,13 @@
     </row>
     <row r="11" spans="1:9" s="11" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A11" s="50"/>
-      <c r="B11" s="67" t="s">
+      <c r="B11" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="79" t="s">
+      <c r="C11" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="138"/>
+      <c r="D11" s="91"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
@@ -2378,13 +2061,13 @@
     </row>
     <row r="12" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A12" s="50"/>
-      <c r="B12" s="66" t="s">
+      <c r="B12" s="59" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="79" t="s">
+      <c r="C12" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="138"/>
+      <c r="D12" s="91"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
@@ -2393,13 +2076,13 @@
     </row>
     <row r="13" spans="1:9" s="11" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A13" s="50"/>
-      <c r="B13" s="66" t="s">
+      <c r="B13" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="79" t="s">
+      <c r="C13" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="138"/>
+      <c r="D13" s="91"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
@@ -2408,13 +2091,13 @@
     </row>
     <row r="14" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A14" s="50"/>
-      <c r="B14" s="66" t="s">
+      <c r="B14" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="79" t="s">
+      <c r="C14" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="140"/>
+      <c r="D14" s="93"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -2423,11 +2106,11 @@
     </row>
     <row r="15" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="50"/>
-      <c r="B15" s="66" t="s">
+      <c r="B15" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="79"/>
-      <c r="D15" s="138"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="91"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
@@ -2436,78 +2119,78 @@
     </row>
     <row r="16" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A16" s="50"/>
-      <c r="B16" s="66" t="s">
+      <c r="B16" s="59" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="79" t="s">
+      <c r="C16" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="157"/>
-      <c r="E16" s="158"/>
-      <c r="F16" s="158"/>
+      <c r="D16" s="110"/>
+      <c r="E16" s="111"/>
+      <c r="F16" s="111"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
       <c r="I16" s="10"/>
     </row>
     <row r="17" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="50"/>
-      <c r="B17" s="66" t="s">
-        <v>197</v>
-      </c>
-      <c r="C17" s="79"/>
-      <c r="D17" s="138"/>
+      <c r="B17" s="59" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="65"/>
+      <c r="D17" s="91"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
       <c r="I17" s="10"/>
     </row>
-    <row r="18" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A18" s="50"/>
-      <c r="B18" s="66" t="s">
-        <v>198</v>
-      </c>
-      <c r="C18" s="79"/>
-      <c r="D18" s="138"/>
+      <c r="B18" s="59" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" s="65"/>
+      <c r="D18" s="91"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
       <c r="I18" s="10"/>
     </row>
-    <row r="19" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" s="11" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A19" s="50"/>
-      <c r="B19" s="68" t="s">
+      <c r="B19" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="79"/>
-      <c r="D19" s="138"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="91"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A20" s="50"/>
-      <c r="B20" s="66" t="s">
+      <c r="B20" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="79"/>
-      <c r="D20" s="138"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="91"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A21" s="50"/>
-      <c r="B21" s="66" t="s">
+      <c r="B21" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="79"/>
-      <c r="D21" s="138"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="91"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -2515,59 +2198,59 @@
       <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:9" s="13" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A22" s="89" t="s">
+      <c r="A22" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="61"/>
-      <c r="C22" s="80" t="s">
+      <c r="B22" s="128"/>
+      <c r="C22" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="139"/>
-      <c r="E22" s="139"/>
-      <c r="F22" s="139"/>
-      <c r="G22" s="139"/>
-      <c r="H22" s="139"/>
-      <c r="I22" s="139"/>
+      <c r="D22" s="92"/>
+      <c r="E22" s="92"/>
+      <c r="F22" s="92"/>
+      <c r="G22" s="92"/>
+      <c r="H22" s="92"/>
+      <c r="I22" s="92"/>
     </row>
     <row r="23" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="51"/>
-      <c r="B23" s="94" t="s">
+      <c r="B23" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="81" t="s">
+      <c r="C23" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="146"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="98"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="83"/>
       <c r="H23" s="14"/>
       <c r="I23" s="15"/>
     </row>
     <row r="24" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="51"/>
-      <c r="B24" s="94" t="s">
+      <c r="B24" s="80" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="81" t="s">
+      <c r="C24" s="67" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="142"/>
+      <c r="D24" s="95"/>
       <c r="E24" s="17"/>
-      <c r="F24" s="99"/>
+      <c r="F24" s="84"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24" s="15"/>
     </row>
     <row r="25" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="51"/>
-      <c r="B25" s="94" t="s">
+      <c r="B25" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="81" t="s">
+      <c r="C25" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="143"/>
+      <c r="D25" s="96"/>
       <c r="E25" s="18"/>
       <c r="F25" s="18"/>
       <c r="G25" s="18"/>
@@ -2576,13 +2259,13 @@
     </row>
     <row r="26" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="51"/>
-      <c r="B26" s="94" t="s">
+      <c r="B26" s="80" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="81" t="s">
+      <c r="C26" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="143"/>
+      <c r="D26" s="96"/>
       <c r="E26" s="18"/>
       <c r="F26" s="18"/>
       <c r="G26" s="18"/>
@@ -2591,13 +2274,13 @@
     </row>
     <row r="27" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A27" s="51"/>
-      <c r="B27" s="94" t="s">
+      <c r="B27" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="81" t="s">
+      <c r="C27" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="143"/>
+      <c r="D27" s="96"/>
       <c r="E27" s="18"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2606,13 +2289,13 @@
     </row>
     <row r="28" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A28" s="51"/>
-      <c r="B28" s="94" t="s">
+      <c r="B28" s="80" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="81" t="s">
+      <c r="C28" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="D28" s="143"/>
+      <c r="D28" s="96"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
       <c r="G28" s="18"/>
@@ -2621,13 +2304,13 @@
     </row>
     <row r="29" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A29" s="51"/>
-      <c r="B29" s="94" t="s">
+      <c r="B29" s="80" t="s">
         <v>56</v>
       </c>
-      <c r="C29" s="81" t="s">
+      <c r="C29" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="143"/>
+      <c r="D29" s="96"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -2636,13 +2319,13 @@
     </row>
     <row r="30" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A30" s="51"/>
-      <c r="B30" s="94" t="s">
+      <c r="B30" s="80" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="81" t="s">
+      <c r="C30" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="141"/>
+      <c r="D30" s="94"/>
       <c r="E30" s="14"/>
       <c r="F30" s="14"/>
       <c r="G30" s="14"/>
@@ -2651,13 +2334,13 @@
     </row>
     <row r="31" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A31" s="51"/>
-      <c r="B31" s="94" t="s">
+      <c r="B31" s="80" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="81" t="s">
+      <c r="C31" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="143"/>
+      <c r="D31" s="96"/>
       <c r="E31" s="18"/>
       <c r="F31" s="19"/>
       <c r="G31" s="19"/>
@@ -2666,13 +2349,13 @@
     </row>
     <row r="32" spans="1:9" s="16" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A32" s="51"/>
-      <c r="B32" s="69" t="s">
+      <c r="B32" s="60" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="81" t="s">
+      <c r="C32" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="144"/>
+      <c r="D32" s="97"/>
       <c r="E32" s="19"/>
       <c r="F32" s="19"/>
       <c r="G32" s="19"/>
@@ -2681,13 +2364,13 @@
     </row>
     <row r="33" spans="1:9" s="16" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A33" s="51"/>
-      <c r="B33" s="69" t="s">
+      <c r="B33" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="C33" s="81" t="s">
+      <c r="C33" s="67" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="145"/>
+      <c r="D33" s="98"/>
       <c r="E33" s="20"/>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -2696,28 +2379,28 @@
     </row>
     <row r="34" spans="1:9" s="16" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A34" s="51"/>
-      <c r="B34" s="69" t="s">
+      <c r="B34" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="81" t="s">
+      <c r="C34" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="D34" s="147"/>
+      <c r="D34" s="100"/>
       <c r="E34" s="21"/>
-      <c r="F34" s="100"/>
+      <c r="F34" s="85"/>
       <c r="G34" s="21"/>
       <c r="H34" s="21"/>
       <c r="I34" s="15"/>
     </row>
     <row r="35" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="52"/>
-      <c r="B35" s="69" t="s">
+      <c r="B35" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="81" t="s">
+      <c r="C35" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="143"/>
+      <c r="D35" s="96"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
       <c r="G35" s="18"/>
@@ -2726,13 +2409,13 @@
     </row>
     <row r="36" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A36" s="51"/>
-      <c r="B36" s="69" t="s">
+      <c r="B36" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="81" t="s">
+      <c r="C36" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="144"/>
+      <c r="D36" s="97"/>
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
@@ -2741,13 +2424,13 @@
     </row>
     <row r="37" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A37" s="51"/>
-      <c r="B37" s="69" t="s">
+      <c r="B37" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="C37" s="81" t="s">
+      <c r="C37" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="D37" s="144"/>
+      <c r="D37" s="97"/>
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
@@ -2755,11 +2438,11 @@
       <c r="I37" s="15"/>
     </row>
     <row r="38" spans="1:9" s="25" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A38" s="90" t="s">
+      <c r="A38" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="B38" s="62"/>
-      <c r="C38" s="82" t="s">
+      <c r="B38" s="129"/>
+      <c r="C38" s="68" t="s">
         <v>77</v>
       </c>
       <c r="D38" s="24"/>
@@ -2771,13 +2454,13 @@
     </row>
     <row r="39" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A39" s="53"/>
-      <c r="B39" s="70" t="s">
-        <v>199</v>
-      </c>
-      <c r="C39" s="83" t="s">
-        <v>200</v>
-      </c>
-      <c r="D39" s="149"/>
+      <c r="B39" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="C39" s="69" t="s">
+        <v>172</v>
+      </c>
+      <c r="D39" s="102"/>
       <c r="E39" s="26"/>
       <c r="F39" s="26"/>
       <c r="G39" s="26"/>
@@ -2786,11 +2469,11 @@
     </row>
     <row r="40" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="53"/>
-      <c r="B40" s="70" t="s">
-        <v>201</v>
-      </c>
-      <c r="C40" s="83"/>
-      <c r="D40" s="149"/>
+      <c r="B40" s="77" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="69"/>
+      <c r="D40" s="102"/>
       <c r="E40" s="26"/>
       <c r="F40" s="26"/>
       <c r="G40" s="26"/>
@@ -2799,37 +2482,37 @@
     </row>
     <row r="41" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="53"/>
-      <c r="B41" s="70" t="s">
-        <v>202</v>
-      </c>
-      <c r="C41" s="83"/>
-      <c r="D41" s="149"/>
+      <c r="B41" s="77" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" s="69"/>
+      <c r="D41" s="102"/>
       <c r="E41" s="26"/>
       <c r="F41" s="26"/>
       <c r="G41" s="26"/>
       <c r="H41" s="26"/>
       <c r="I41" s="27"/>
     </row>
-    <row r="42" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A42" s="53"/>
-      <c r="B42" s="70" t="s">
-        <v>203</v>
-      </c>
-      <c r="C42" s="83"/>
-      <c r="D42" s="149"/>
+      <c r="B42" s="77" t="s">
+        <v>175</v>
+      </c>
+      <c r="C42" s="69"/>
+      <c r="D42" s="102"/>
       <c r="E42" s="26"/>
       <c r="F42" s="26"/>
       <c r="G42" s="26"/>
       <c r="H42" s="26"/>
       <c r="I42" s="27"/>
     </row>
-    <row r="43" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A43" s="53"/>
-      <c r="B43" s="70" t="s">
-        <v>204</v>
-      </c>
-      <c r="C43" s="83"/>
-      <c r="D43" s="149"/>
+      <c r="B43" s="77" t="s">
+        <v>176</v>
+      </c>
+      <c r="C43" s="69"/>
+      <c r="D43" s="102"/>
       <c r="E43" s="26"/>
       <c r="F43" s="26"/>
       <c r="G43" s="26"/>
@@ -2838,11 +2521,11 @@
     </row>
     <row r="44" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="53"/>
-      <c r="B44" s="70" t="s">
-        <v>205</v>
-      </c>
-      <c r="C44" s="83"/>
-      <c r="D44" s="149"/>
+      <c r="B44" s="77" t="s">
+        <v>177</v>
+      </c>
+      <c r="C44" s="69"/>
+      <c r="D44" s="102"/>
       <c r="E44" s="26"/>
       <c r="F44" s="26"/>
       <c r="G44" s="26"/>
@@ -2851,106 +2534,106 @@
     </row>
     <row r="45" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A45" s="53"/>
-      <c r="B45" s="71" t="s">
-        <v>206</v>
-      </c>
-      <c r="C45" s="83" t="s">
-        <v>212</v>
-      </c>
-      <c r="D45" s="149"/>
-      <c r="E45" s="159"/>
+      <c r="B45" s="130" t="s">
+        <v>178</v>
+      </c>
+      <c r="C45" s="69" t="s">
+        <v>184</v>
+      </c>
+      <c r="D45" s="102"/>
+      <c r="E45" s="112"/>
       <c r="F45" s="26"/>
-      <c r="G45" s="159"/>
-      <c r="H45" s="159"/>
+      <c r="G45" s="112"/>
+      <c r="H45" s="112"/>
       <c r="I45" s="27"/>
     </row>
     <row r="46" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="53"/>
-      <c r="B46" s="71" t="s">
-        <v>207</v>
-      </c>
-      <c r="C46" s="83"/>
-      <c r="D46" s="149"/>
-      <c r="E46" s="159"/>
+      <c r="B46" s="130" t="s">
+        <v>179</v>
+      </c>
+      <c r="C46" s="69"/>
+      <c r="D46" s="102"/>
+      <c r="E46" s="112"/>
       <c r="F46" s="26"/>
-      <c r="G46" s="159"/>
-      <c r="H46" s="159"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="112"/>
       <c r="I46" s="27"/>
     </row>
     <row r="47" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="53"/>
-      <c r="B47" s="71" t="s">
-        <v>208</v>
-      </c>
-      <c r="C47" s="83"/>
-      <c r="D47" s="149"/>
-      <c r="E47" s="159"/>
+      <c r="B47" s="130" t="s">
+        <v>180</v>
+      </c>
+      <c r="C47" s="69"/>
+      <c r="D47" s="102"/>
+      <c r="E47" s="112"/>
       <c r="F47" s="26"/>
-      <c r="G47" s="159"/>
-      <c r="H47" s="159"/>
+      <c r="G47" s="112"/>
+      <c r="H47" s="112"/>
       <c r="I47" s="27"/>
     </row>
-    <row r="48" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A48" s="53"/>
-      <c r="B48" s="71" t="s">
-        <v>209</v>
-      </c>
-      <c r="C48" s="83"/>
-      <c r="D48" s="149"/>
-      <c r="E48" s="159"/>
+      <c r="B48" s="130" t="s">
+        <v>181</v>
+      </c>
+      <c r="C48" s="69"/>
+      <c r="D48" s="102"/>
+      <c r="E48" s="112"/>
       <c r="F48" s="26"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="159"/>
+      <c r="G48" s="112"/>
+      <c r="H48" s="112"/>
       <c r="I48" s="27"/>
     </row>
-    <row r="49" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:47" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A49" s="53"/>
-      <c r="B49" s="71" t="s">
-        <v>210</v>
-      </c>
-      <c r="C49" s="83"/>
-      <c r="D49" s="149"/>
-      <c r="E49" s="159"/>
+      <c r="B49" s="130" t="s">
+        <v>182</v>
+      </c>
+      <c r="C49" s="69"/>
+      <c r="D49" s="102"/>
+      <c r="E49" s="112"/>
       <c r="F49" s="26"/>
-      <c r="G49" s="159"/>
-      <c r="H49" s="159"/>
+      <c r="G49" s="112"/>
+      <c r="H49" s="112"/>
       <c r="I49" s="27"/>
     </row>
     <row r="50" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="53"/>
-      <c r="B50" s="71" t="s">
-        <v>211</v>
-      </c>
-      <c r="C50" s="83"/>
-      <c r="D50" s="149"/>
-      <c r="E50" s="159"/>
+      <c r="B50" s="130" t="s">
+        <v>183</v>
+      </c>
+      <c r="C50" s="69"/>
+      <c r="D50" s="102"/>
+      <c r="E50" s="112"/>
       <c r="F50" s="26"/>
-      <c r="G50" s="159"/>
-      <c r="H50" s="159"/>
+      <c r="G50" s="112"/>
+      <c r="H50" s="112"/>
       <c r="I50" s="27"/>
     </row>
     <row r="51" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="53"/>
-      <c r="B51" s="70" t="s">
+      <c r="B51" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C51" s="83"/>
-      <c r="D51" s="149"/>
-      <c r="E51" s="149"/>
-      <c r="F51" s="149"/>
-      <c r="G51" s="149"/>
-      <c r="H51" s="149"/>
+      <c r="C51" s="69"/>
+      <c r="D51" s="102"/>
+      <c r="E51" s="102"/>
+      <c r="F51" s="102"/>
+      <c r="G51" s="102"/>
+      <c r="H51" s="102"/>
       <c r="I51" s="27"/>
     </row>
     <row r="52" spans="1:47" s="28" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A52" s="53"/>
-      <c r="B52" s="91" t="s">
+      <c r="B52" s="77" t="s">
         <v>80</v>
       </c>
-      <c r="C52" s="83" t="s">
+      <c r="C52" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="D52" s="149"/>
+      <c r="D52" s="102"/>
       <c r="E52" s="26"/>
       <c r="F52" s="26"/>
       <c r="G52" s="26"/>
@@ -2958,14 +2641,14 @@
       <c r="I52" s="27"/>
     </row>
     <row r="53" spans="1:47" s="31" customFormat="1" ht="65" x14ac:dyDescent="0.3">
-      <c r="A53" s="97" t="s">
+      <c r="A53" s="82" t="s">
         <v>82</v>
       </c>
-      <c r="B53" s="63"/>
-      <c r="C53" s="84" t="s">
+      <c r="B53" s="131"/>
+      <c r="C53" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="D53" s="150"/>
+      <c r="D53" s="103"/>
       <c r="E53" s="29"/>
       <c r="F53" s="29"/>
       <c r="G53" s="29"/>
@@ -2974,13 +2657,13 @@
     </row>
     <row r="54" spans="1:47" s="34" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A54" s="54"/>
-      <c r="B54" s="72" t="s">
+      <c r="B54" s="132" t="s">
         <v>84</v>
       </c>
-      <c r="C54" s="85" t="s">
+      <c r="C54" s="71" t="s">
         <v>85</v>
       </c>
-      <c r="D54" s="151"/>
+      <c r="D54" s="104"/>
       <c r="E54" s="32"/>
       <c r="F54" s="32"/>
       <c r="G54" s="32"/>
@@ -2989,13 +2672,13 @@
     </row>
     <row r="55" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A55" s="54"/>
-      <c r="B55" s="72" t="s">
+      <c r="B55" s="132" t="s">
         <v>86</v>
       </c>
-      <c r="C55" s="85" t="s">
+      <c r="C55" s="71" t="s">
         <v>87</v>
       </c>
-      <c r="D55" s="152"/>
+      <c r="D55" s="105"/>
       <c r="E55" s="35"/>
       <c r="F55" s="35"/>
       <c r="G55" s="35"/>
@@ -3004,28 +2687,28 @@
     </row>
     <row r="56" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A56" s="54"/>
-      <c r="B56" s="72" t="s">
+      <c r="B56" s="132" t="s">
         <v>88</v>
       </c>
-      <c r="C56" s="85" t="s">
+      <c r="C56" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="D56" s="153"/>
-      <c r="E56" s="148"/>
-      <c r="F56" s="148"/>
-      <c r="G56" s="148"/>
-      <c r="H56" s="148"/>
+      <c r="D56" s="106"/>
+      <c r="E56" s="101"/>
+      <c r="F56" s="101"/>
+      <c r="G56" s="101"/>
+      <c r="H56" s="101"/>
       <c r="I56" s="33"/>
     </row>
     <row r="57" spans="1:47" s="34" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A57" s="54"/>
-      <c r="B57" s="72" t="s">
+      <c r="B57" s="132" t="s">
         <v>91</v>
       </c>
-      <c r="C57" s="85" t="s">
+      <c r="C57" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="D57" s="154"/>
+      <c r="D57" s="107"/>
       <c r="E57" s="36"/>
       <c r="F57" s="36"/>
       <c r="G57" s="36"/>
@@ -3034,13 +2717,13 @@
     </row>
     <row r="58" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A58" s="54"/>
-      <c r="B58" s="72" t="s">
+      <c r="B58" s="132" t="s">
         <v>93</v>
       </c>
-      <c r="C58" s="85" t="s">
+      <c r="C58" s="71" t="s">
         <v>94</v>
       </c>
-      <c r="D58" s="152"/>
+      <c r="D58" s="105"/>
       <c r="E58" s="35"/>
       <c r="F58" s="35"/>
       <c r="G58" s="35"/>
@@ -3049,25 +2732,25 @@
     </row>
     <row r="59" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A59" s="54"/>
-      <c r="B59" s="72" t="s">
+      <c r="B59" s="132" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="85" t="s">
+      <c r="C59" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="D59" s="148"/>
-      <c r="E59" s="148"/>
-      <c r="F59" s="148"/>
-      <c r="G59" s="148"/>
-      <c r="H59" s="148"/>
+      <c r="D59" s="101"/>
+      <c r="E59" s="101"/>
+      <c r="F59" s="101"/>
+      <c r="G59" s="101"/>
+      <c r="H59" s="101"/>
       <c r="I59" s="33"/>
     </row>
     <row r="60" spans="1:47" s="38" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A60" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="B60" s="64"/>
-      <c r="C60" s="86" t="s">
+      <c r="B60" s="133"/>
+      <c r="C60" s="72" t="s">
         <v>99</v>
       </c>
       <c r="D60" s="37"/>
@@ -3079,13 +2762,13 @@
     </row>
     <row r="61" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="56"/>
-      <c r="B61" s="73" t="s">
+      <c r="B61" s="134" t="s">
         <v>100</v>
       </c>
-      <c r="C61" s="87" t="s">
+      <c r="C61" s="73" t="s">
         <v>101</v>
       </c>
-      <c r="D61" s="155"/>
+      <c r="D61" s="108"/>
       <c r="E61" s="39"/>
       <c r="F61" s="39"/>
       <c r="G61" s="39"/>
@@ -3094,47 +2777,47 @@
     </row>
     <row r="62" spans="1:47" s="41" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A62" s="56"/>
-      <c r="B62" s="73" t="s">
+      <c r="B62" s="134" t="s">
         <v>102</v>
       </c>
-      <c r="C62" s="87" t="s">
+      <c r="C62" s="73" t="s">
         <v>103</v>
       </c>
-      <c r="D62" s="155"/>
+      <c r="D62" s="108"/>
       <c r="E62" s="39"/>
       <c r="F62" s="39"/>
       <c r="G62" s="39"/>
       <c r="H62" s="39"/>
       <c r="I62" s="40"/>
     </row>
-    <row r="63" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:47" s="41" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A63" s="56"/>
-      <c r="B63" s="73" t="s">
+      <c r="B63" s="134" t="s">
         <v>104</v>
       </c>
-      <c r="C63" s="87" t="s">
+      <c r="C63" s="73" t="s">
         <v>105</v>
       </c>
-      <c r="D63" s="155"/>
-      <c r="E63" s="155"/>
-      <c r="F63" s="155"/>
-      <c r="G63" s="155"/>
-      <c r="H63" s="155"/>
+      <c r="D63" s="108"/>
+      <c r="E63" s="108"/>
+      <c r="F63" s="108"/>
+      <c r="G63" s="108"/>
+      <c r="H63" s="108"/>
       <c r="I63" s="56"/>
     </row>
-    <row r="64" spans="1:47" s="42" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:47" s="42" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A64" s="56"/>
-      <c r="B64" s="73" t="s">
+      <c r="B64" s="134" t="s">
         <v>106</v>
       </c>
-      <c r="C64" s="87" t="s">
+      <c r="C64" s="73" t="s">
         <v>107</v>
       </c>
-      <c r="D64" s="155"/>
-      <c r="E64" s="155"/>
-      <c r="F64" s="155"/>
-      <c r="G64" s="155"/>
-      <c r="H64" s="155"/>
+      <c r="D64" s="108"/>
+      <c r="E64" s="108"/>
+      <c r="F64" s="108"/>
+      <c r="G64" s="108"/>
+      <c r="H64" s="108"/>
       <c r="I64" s="56"/>
       <c r="J64" s="56"/>
       <c r="K64" s="56"/>
@@ -3175,17 +2858,17 @@
       <c r="AT64" s="56"/>
       <c r="AU64" s="56"/>
     </row>
-    <row r="65" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A65" s="56"/>
-      <c r="B65" s="73" t="s">
+      <c r="B65" s="134" t="s">
         <v>108</v>
       </c>
-      <c r="C65" s="87"/>
-      <c r="D65" s="155"/>
-      <c r="E65" s="155"/>
-      <c r="F65" s="155"/>
-      <c r="G65" s="155"/>
-      <c r="H65" s="155"/>
+      <c r="C65" s="73"/>
+      <c r="D65" s="108"/>
+      <c r="E65" s="108"/>
+      <c r="F65" s="108"/>
+      <c r="G65" s="108"/>
+      <c r="H65" s="108"/>
       <c r="I65" s="56"/>
       <c r="J65" s="56"/>
       <c r="K65" s="56"/>
@@ -3226,17 +2909,17 @@
       <c r="AT65" s="56"/>
       <c r="AU65" s="56"/>
     </row>
-    <row r="66" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A66" s="56"/>
-      <c r="B66" s="73" t="s">
+      <c r="B66" s="134" t="s">
         <v>109</v>
       </c>
-      <c r="C66" s="87"/>
-      <c r="D66" s="155"/>
-      <c r="E66" s="155"/>
-      <c r="F66" s="155"/>
-      <c r="G66" s="155"/>
-      <c r="H66" s="155"/>
+      <c r="C66" s="73"/>
+      <c r="D66" s="108"/>
+      <c r="E66" s="108"/>
+      <c r="F66" s="108"/>
+      <c r="G66" s="108"/>
+      <c r="H66" s="108"/>
       <c r="I66" s="56"/>
       <c r="J66" s="56"/>
       <c r="K66" s="56"/>
@@ -3277,17 +2960,17 @@
       <c r="AT66" s="56"/>
       <c r="AU66" s="56"/>
     </row>
-    <row r="67" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:47" s="45" customFormat="1" ht="56" x14ac:dyDescent="0.3">
       <c r="A67" s="56"/>
-      <c r="B67" s="73" t="s">
+      <c r="B67" s="134" t="s">
         <v>110</v>
       </c>
-      <c r="C67" s="87"/>
-      <c r="D67" s="155"/>
-      <c r="E67" s="155"/>
-      <c r="F67" s="155"/>
-      <c r="G67" s="155"/>
-      <c r="H67" s="155"/>
+      <c r="C67" s="73"/>
+      <c r="D67" s="108"/>
+      <c r="E67" s="108"/>
+      <c r="F67" s="108"/>
+      <c r="G67" s="108"/>
+      <c r="H67" s="108"/>
       <c r="I67" s="56"/>
       <c r="J67" s="56"/>
       <c r="K67" s="56"/>
@@ -3328,17 +3011,17 @@
       <c r="AT67" s="56"/>
       <c r="AU67" s="56"/>
     </row>
-    <row r="68" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A68" s="56"/>
-      <c r="B68" s="73" t="s">
+      <c r="B68" s="134" t="s">
         <v>111</v>
       </c>
-      <c r="C68" s="87"/>
-      <c r="D68" s="155"/>
-      <c r="E68" s="155"/>
-      <c r="F68" s="155"/>
-      <c r="G68" s="155"/>
-      <c r="H68" s="155"/>
+      <c r="C68" s="73"/>
+      <c r="D68" s="108"/>
+      <c r="E68" s="108"/>
+      <c r="F68" s="108"/>
+      <c r="G68" s="108"/>
+      <c r="H68" s="108"/>
       <c r="I68" s="56"/>
       <c r="J68" s="56"/>
       <c r="K68" s="56"/>
@@ -3379,67 +3062,67 @@
       <c r="AT68" s="56"/>
       <c r="AU68" s="56"/>
     </row>
-    <row r="69" spans="1:47" s="105" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="101" t="s">
+    <row r="69" spans="1:47" s="89" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="86" t="s">
         <v>162</v>
       </c>
-      <c r="B69" s="102"/>
-      <c r="C69" s="103"/>
-      <c r="D69" s="104"/>
-      <c r="E69" s="104"/>
-      <c r="F69" s="104"/>
-      <c r="G69" s="104"/>
-      <c r="H69" s="104"/>
-      <c r="I69" s="104"/>
-    </row>
-    <row r="70" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="B69" s="135"/>
+      <c r="C69" s="87"/>
+      <c r="D69" s="88"/>
+      <c r="E69" s="88"/>
+      <c r="F69" s="88"/>
+      <c r="G69" s="88"/>
+      <c r="H69" s="88"/>
+      <c r="I69" s="88"/>
+    </row>
+    <row r="70" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A70" s="57"/>
-      <c r="B70" s="74" t="s">
+      <c r="B70" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="C70" s="88" t="s">
+      <c r="C70" s="74" t="s">
         <v>113</v>
       </c>
-      <c r="D70" s="156"/>
-      <c r="E70" s="156"/>
-      <c r="F70" s="156"/>
-      <c r="G70" s="156"/>
+      <c r="D70" s="109"/>
+      <c r="E70" s="109"/>
+      <c r="F70" s="109"/>
+      <c r="G70" s="109"/>
       <c r="H70" s="43"/>
       <c r="I70" s="44"/>
     </row>
-    <row r="71" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A71" s="57"/>
-      <c r="B71" s="74" t="s">
+      <c r="B71" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="C71" s="88"/>
-      <c r="D71" s="156"/>
+      <c r="C71" s="74"/>
+      <c r="D71" s="109"/>
       <c r="E71" s="43"/>
       <c r="F71" s="43"/>
       <c r="G71" s="43"/>
       <c r="H71" s="43"/>
       <c r="I71" s="44"/>
     </row>
-    <row r="72" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A72" s="57"/>
-      <c r="B72" s="74" t="s">
+      <c r="B72" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="C72" s="88"/>
-      <c r="D72" s="156"/>
+      <c r="C72" s="74"/>
+      <c r="D72" s="109"/>
       <c r="E72" s="43"/>
       <c r="F72" s="43"/>
       <c r="G72" s="43"/>
       <c r="H72" s="43"/>
       <c r="I72" s="44"/>
     </row>
-    <row r="73" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:47" s="45" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A73" s="57"/>
-      <c r="B73" s="75" t="s">
+      <c r="B73" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="C73" s="88"/>
-      <c r="D73" s="156"/>
+      <c r="C73" s="74"/>
+      <c r="D73" s="109"/>
       <c r="E73" s="43"/>
       <c r="F73" s="43"/>
       <c r="G73" s="43"/>
@@ -3448,11 +3131,11 @@
     </row>
     <row r="74" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A74" s="57"/>
-      <c r="B74" s="75" t="s">
+      <c r="B74" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="C74" s="88"/>
-      <c r="D74" s="156"/>
+      <c r="C74" s="74"/>
+      <c r="D74" s="109"/>
       <c r="E74" s="43"/>
       <c r="F74" s="43"/>
       <c r="G74" s="43"/>
@@ -3461,13 +3144,13 @@
     </row>
     <row r="75" spans="1:47" s="45" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A75" s="57"/>
-      <c r="B75" s="74" t="s">
+      <c r="B75" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="C75" s="88" t="s">
+      <c r="C75" s="74" t="s">
         <v>119</v>
       </c>
-      <c r="D75" s="156"/>
+      <c r="D75" s="109"/>
       <c r="E75" s="43"/>
       <c r="F75" s="43"/>
       <c r="G75" s="43"/>
@@ -3476,13 +3159,13 @@
     </row>
     <row r="76" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A76" s="57"/>
-      <c r="B76" s="74" t="s">
-        <v>216</v>
-      </c>
-      <c r="C76" s="88" t="s">
-        <v>217</v>
-      </c>
-      <c r="D76" s="156"/>
+      <c r="B76" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="C76" s="74" t="s">
+        <v>189</v>
+      </c>
+      <c r="D76" s="109"/>
       <c r="E76" s="43"/>
       <c r="F76" s="43"/>
       <c r="G76" s="43"/>
@@ -3491,13 +3174,13 @@
     </row>
     <row r="77" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A77" s="57"/>
-      <c r="B77" s="74" t="s">
-        <v>213</v>
-      </c>
-      <c r="C77" s="88" t="s">
-        <v>218</v>
-      </c>
-      <c r="D77" s="156"/>
+      <c r="B77" s="61" t="s">
+        <v>185</v>
+      </c>
+      <c r="C77" s="74" t="s">
+        <v>190</v>
+      </c>
+      <c r="D77" s="109"/>
       <c r="E77" s="43"/>
       <c r="F77" s="43"/>
       <c r="G77" s="43"/>
@@ -3506,13 +3189,13 @@
     </row>
     <row r="78" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="57"/>
-      <c r="B78" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="C78" s="88" t="s">
-        <v>215</v>
-      </c>
-      <c r="D78" s="156"/>
+      <c r="B78" s="61" t="s">
+        <v>186</v>
+      </c>
+      <c r="C78" s="74" t="s">
+        <v>187</v>
+      </c>
+      <c r="D78" s="109"/>
       <c r="E78" s="43"/>
       <c r="F78" s="43"/>
       <c r="G78" s="43"/>
@@ -3521,167 +3204,197 @@
     </row>
     <row r="79" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="57"/>
-      <c r="B79" s="74" t="s">
+      <c r="B79" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="C79" s="88" t="s">
+      <c r="C79" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="D79" s="156"/>
+      <c r="D79" s="109"/>
       <c r="E79" s="43"/>
       <c r="F79" s="43"/>
       <c r="G79" s="43"/>
       <c r="H79" s="43"/>
       <c r="I79" s="44"/>
     </row>
-    <row r="80" spans="1:47" s="167" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="163" t="s">
-        <v>222</v>
-      </c>
-      <c r="B80" s="164"/>
-      <c r="C80" s="165"/>
-      <c r="D80" s="166"/>
-      <c r="E80" s="166"/>
-      <c r="F80" s="166"/>
-      <c r="G80" s="166"/>
-      <c r="H80" s="166"/>
-      <c r="I80" s="166"/>
-    </row>
-    <row r="81" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="160"/>
-      <c r="B81" s="168" t="s">
-        <v>223</v>
-      </c>
-      <c r="C81" s="169" t="s">
-        <v>229</v>
-      </c>
-      <c r="D81" s="170"/>
-      <c r="E81" s="170"/>
-      <c r="F81" s="170"/>
-      <c r="G81" s="170"/>
-      <c r="H81" s="170"/>
-      <c r="I81" s="161"/>
-    </row>
-    <row r="82" spans="1:9" s="162" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A82" s="160"/>
-      <c r="B82" s="168" t="s">
-        <v>234</v>
-      </c>
-      <c r="C82" s="169" t="s">
-        <v>235</v>
-      </c>
-      <c r="D82" s="170"/>
-      <c r="E82" s="170"/>
-      <c r="F82" s="170"/>
-      <c r="G82" s="170"/>
-      <c r="H82" s="170"/>
-      <c r="I82" s="161"/>
-    </row>
-    <row r="83" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="160"/>
-      <c r="B83" s="168" t="s">
-        <v>230</v>
-      </c>
-      <c r="C83" s="169"/>
-      <c r="D83" s="170"/>
-      <c r="E83" s="170"/>
-      <c r="F83" s="170"/>
-      <c r="G83" s="170"/>
-      <c r="H83" s="170"/>
-      <c r="I83" s="161"/>
-    </row>
-    <row r="84" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="160"/>
-      <c r="B84" s="168" t="s">
-        <v>231</v>
-      </c>
-      <c r="C84" s="169"/>
-      <c r="D84" s="170"/>
-      <c r="E84" s="170"/>
-      <c r="F84" s="170"/>
-      <c r="G84" s="170"/>
-      <c r="H84" s="170"/>
-      <c r="I84" s="161"/>
-    </row>
-    <row r="85" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="160"/>
-      <c r="B85" s="168" t="s">
-        <v>224</v>
-      </c>
-      <c r="C85" s="169"/>
-      <c r="D85" s="170"/>
-      <c r="E85" s="170"/>
-      <c r="F85" s="170"/>
-      <c r="G85" s="170"/>
-      <c r="H85" s="170"/>
-      <c r="I85" s="161"/>
-    </row>
-    <row r="86" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="160"/>
-      <c r="B86" s="168" t="s">
-        <v>225</v>
-      </c>
-      <c r="C86" s="169"/>
-      <c r="D86" s="170"/>
-      <c r="E86" s="170"/>
-      <c r="F86" s="170"/>
-      <c r="G86" s="170"/>
-      <c r="H86" s="170"/>
-      <c r="I86" s="161"/>
-    </row>
-    <row r="87" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="160"/>
-      <c r="B87" s="168" t="s">
-        <v>226</v>
-      </c>
-      <c r="C87" s="169"/>
-      <c r="D87" s="170"/>
-      <c r="E87" s="170"/>
-      <c r="F87" s="170"/>
-      <c r="G87" s="170"/>
-      <c r="H87" s="170"/>
-      <c r="I87" s="161"/>
-    </row>
-    <row r="88" spans="1:9" s="162" customFormat="1" ht="31" x14ac:dyDescent="0.3">
-      <c r="A88" s="160"/>
-      <c r="B88" s="171" t="s">
-        <v>227</v>
-      </c>
-      <c r="C88" s="169"/>
-      <c r="D88" s="170"/>
-      <c r="E88" s="170"/>
-      <c r="F88" s="170"/>
-      <c r="G88" s="170"/>
-      <c r="H88" s="170"/>
-      <c r="I88" s="161"/>
-    </row>
-    <row r="89" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="160"/>
-      <c r="B89" s="168" t="s">
-        <v>228</v>
-      </c>
-      <c r="C89" s="169"/>
-      <c r="D89" s="170"/>
-      <c r="E89" s="170"/>
-      <c r="F89" s="170"/>
-      <c r="G89" s="170"/>
-      <c r="H89" s="170"/>
-      <c r="I89" s="161"/>
-    </row>
-    <row r="90" spans="1:9" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="160"/>
-      <c r="B90" s="172" t="s">
-        <v>232</v>
-      </c>
-      <c r="C90" s="169" t="s">
-        <v>233</v>
-      </c>
-      <c r="D90" s="170"/>
-      <c r="E90" s="170"/>
-      <c r="F90" s="170"/>
-      <c r="G90" s="170"/>
-      <c r="H90" s="170"/>
-      <c r="I90" s="161"/>
+    <row r="80" spans="1:47" s="119" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="116" t="s">
+        <v>194</v>
+      </c>
+      <c r="B80" s="136"/>
+      <c r="C80" s="117"/>
+      <c r="D80" s="118"/>
+      <c r="E80" s="118"/>
+      <c r="F80" s="118"/>
+      <c r="G80" s="118"/>
+      <c r="H80" s="118"/>
+      <c r="I80" s="118"/>
+    </row>
+    <row r="81" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="113"/>
+      <c r="B81" s="122" t="s">
+        <v>195</v>
+      </c>
+      <c r="C81" s="120" t="s">
+        <v>201</v>
+      </c>
+      <c r="D81" s="121"/>
+      <c r="E81" s="121"/>
+      <c r="F81" s="121"/>
+      <c r="G81" s="121"/>
+      <c r="H81" s="121"/>
+      <c r="I81" s="114"/>
+    </row>
+    <row r="82" spans="1:9" s="115" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A82" s="113"/>
+      <c r="B82" s="122" t="s">
+        <v>206</v>
+      </c>
+      <c r="C82" s="120" t="s">
+        <v>207</v>
+      </c>
+      <c r="D82" s="121"/>
+      <c r="E82" s="121"/>
+      <c r="F82" s="121"/>
+      <c r="G82" s="121"/>
+      <c r="H82" s="121"/>
+      <c r="I82" s="114"/>
+    </row>
+    <row r="83" spans="1:9" s="115" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A83" s="113"/>
+      <c r="B83" s="122" t="s">
+        <v>211</v>
+      </c>
+      <c r="C83" s="120" t="s">
+        <v>213</v>
+      </c>
+      <c r="D83" s="121"/>
+      <c r="E83" s="121"/>
+      <c r="F83" s="121"/>
+      <c r="G83" s="121"/>
+      <c r="H83" s="121"/>
+      <c r="I83" s="114"/>
+    </row>
+    <row r="84" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="113"/>
+      <c r="B84" s="138" t="s">
+        <v>212</v>
+      </c>
+      <c r="C84" s="115" t="s">
+        <v>214</v>
+      </c>
+      <c r="D84" s="121"/>
+      <c r="E84" s="121"/>
+      <c r="F84" s="121"/>
+      <c r="G84" s="121"/>
+      <c r="H84" s="121"/>
+      <c r="I84" s="114"/>
+    </row>
+    <row r="85" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="113"/>
+      <c r="B85" s="122" t="s">
+        <v>202</v>
+      </c>
+      <c r="C85" s="120"/>
+      <c r="D85" s="121"/>
+      <c r="E85" s="121"/>
+      <c r="F85" s="121"/>
+      <c r="G85" s="121"/>
+      <c r="H85" s="121"/>
+      <c r="I85" s="114"/>
+    </row>
+    <row r="86" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="113"/>
+      <c r="B86" s="122" t="s">
+        <v>203</v>
+      </c>
+      <c r="C86" s="120"/>
+      <c r="D86" s="121"/>
+      <c r="E86" s="121"/>
+      <c r="F86" s="121"/>
+      <c r="G86" s="121"/>
+      <c r="H86" s="121"/>
+      <c r="I86" s="114"/>
+    </row>
+    <row r="87" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="113"/>
+      <c r="B87" s="122" t="s">
+        <v>196</v>
+      </c>
+      <c r="C87" s="120"/>
+      <c r="D87" s="121"/>
+      <c r="E87" s="121"/>
+      <c r="F87" s="121"/>
+      <c r="G87" s="121"/>
+      <c r="H87" s="121"/>
+      <c r="I87" s="114"/>
+    </row>
+    <row r="88" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="113"/>
+      <c r="B88" s="122" t="s">
+        <v>197</v>
+      </c>
+      <c r="C88" s="120"/>
+      <c r="D88" s="121"/>
+      <c r="E88" s="121"/>
+      <c r="F88" s="121"/>
+      <c r="G88" s="121"/>
+      <c r="H88" s="121"/>
+      <c r="I88" s="114"/>
+    </row>
+    <row r="89" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="113"/>
+      <c r="B89" s="122" t="s">
+        <v>198</v>
+      </c>
+      <c r="C89" s="120"/>
+      <c r="D89" s="121"/>
+      <c r="E89" s="121"/>
+      <c r="F89" s="121"/>
+      <c r="G89" s="121"/>
+      <c r="H89" s="121"/>
+      <c r="I89" s="114"/>
+    </row>
+    <row r="90" spans="1:9" s="115" customFormat="1" ht="45" x14ac:dyDescent="0.3">
+      <c r="A90" s="113"/>
+      <c r="B90" s="122" t="s">
+        <v>199</v>
+      </c>
+      <c r="C90" s="120"/>
+      <c r="D90" s="121"/>
+      <c r="E90" s="121"/>
+      <c r="F90" s="121"/>
+      <c r="G90" s="121"/>
+      <c r="H90" s="121"/>
+      <c r="I90" s="114"/>
+    </row>
+    <row r="91" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="113"/>
+      <c r="B91" s="122" t="s">
+        <v>200</v>
+      </c>
+      <c r="C91" s="120"/>
+      <c r="D91" s="121"/>
+      <c r="E91" s="121"/>
+      <c r="F91" s="121"/>
+      <c r="G91" s="121"/>
+      <c r="H91" s="121"/>
+      <c r="I91" s="114"/>
+    </row>
+    <row r="92" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="113"/>
+      <c r="B92" s="137" t="s">
+        <v>204</v>
+      </c>
+      <c r="C92" s="120" t="s">
+        <v>205</v>
+      </c>
+      <c r="D92" s="121"/>
+      <c r="E92" s="121"/>
+      <c r="F92" s="121"/>
+      <c r="G92" s="121"/>
+      <c r="H92" s="121"/>
+      <c r="I92" s="114"/>
     </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
@@ -3703,370 +3416,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C559A218-9020-4822-8346-393500FE199B}">
-  <dimension ref="A1:I69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" style="58" customWidth="1"/>
-    <col min="3" max="3" width="39.1640625" style="65" customWidth="1"/>
-    <col min="4" max="8" width="32.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="58" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="65" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="65" x14ac:dyDescent="0.3">
-      <c r="C2" s="65" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" s="114" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A3" s="112" t="s">
-        <v>164</v>
-      </c>
-      <c r="B3" s="115"/>
-      <c r="C3" s="116" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="113"/>
-      <c r="E3" s="113"/>
-      <c r="F3" s="113"/>
-      <c r="G3" s="113"/>
-      <c r="H3" s="113"/>
-      <c r="I3" s="113"/>
-    </row>
-    <row r="4" spans="1:9" s="108" customFormat="1" ht="169" x14ac:dyDescent="0.3">
-      <c r="A4" s="107"/>
-      <c r="B4" s="109" t="s">
-        <v>184</v>
-      </c>
-      <c r="C4" s="110" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" s="111"/>
-      <c r="E4" s="111"/>
-      <c r="F4" s="111"/>
-      <c r="G4" s="111"/>
-      <c r="H4" s="111"/>
-      <c r="I4" s="106"/>
-    </row>
-    <row r="5" spans="1:9" s="108" customFormat="1" ht="78" x14ac:dyDescent="0.3">
-      <c r="A5" s="107"/>
-      <c r="B5" s="109" t="s">
-        <v>165</v>
-      </c>
-      <c r="C5" s="110" t="s">
-        <v>167</v>
-      </c>
-      <c r="D5" s="111"/>
-      <c r="E5" s="111"/>
-      <c r="F5" s="111"/>
-      <c r="G5" s="111"/>
-      <c r="H5" s="111"/>
-      <c r="I5" s="106"/>
-    </row>
-    <row r="6" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A6" s="107"/>
-      <c r="B6" s="109" t="s">
-        <v>193</v>
-      </c>
-      <c r="C6" s="110" t="s">
-        <v>194</v>
-      </c>
-      <c r="D6" s="111"/>
-      <c r="E6" s="111"/>
-      <c r="F6" s="111"/>
-      <c r="G6" s="111"/>
-      <c r="H6" s="111"/>
-      <c r="I6" s="106"/>
-    </row>
-    <row r="7" spans="1:9" s="108" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A7" s="107"/>
-      <c r="B7" s="109" t="s">
-        <v>192</v>
-      </c>
-      <c r="C7" s="110" t="s">
-        <v>195</v>
-      </c>
-      <c r="D7" s="111"/>
-      <c r="E7" s="111"/>
-      <c r="F7" s="111"/>
-      <c r="G7" s="111"/>
-      <c r="H7" s="111"/>
-      <c r="I7" s="106"/>
-    </row>
-    <row r="8" spans="1:9" s="108" customFormat="1" ht="52" x14ac:dyDescent="0.3">
-      <c r="A8" s="107"/>
-      <c r="B8" s="109" t="s">
-        <v>166</v>
-      </c>
-      <c r="C8" s="110" t="s">
-        <v>168</v>
-      </c>
-      <c r="D8" s="134"/>
-      <c r="E8" s="111"/>
-      <c r="F8" s="111"/>
-      <c r="G8" s="111"/>
-      <c r="H8" s="111"/>
-      <c r="I8" s="106"/>
-    </row>
-    <row r="9" spans="1:9" s="129" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A9" s="125" t="s">
-        <v>169</v>
-      </c>
-      <c r="B9" s="126"/>
-      <c r="C9" s="127" t="s">
-        <v>171</v>
-      </c>
-      <c r="D9" s="128"/>
-      <c r="E9" s="128"/>
-      <c r="F9" s="128"/>
-      <c r="G9" s="128"/>
-      <c r="H9" s="128"/>
-      <c r="I9" s="128"/>
-    </row>
-    <row r="10" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="117"/>
-      <c r="B10" s="121" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" s="118" t="s">
-        <v>172</v>
-      </c>
-      <c r="D10" s="122"/>
-      <c r="E10" s="123"/>
-      <c r="F10" s="123"/>
-      <c r="G10" s="123"/>
-      <c r="H10" s="123"/>
-      <c r="I10" s="119"/>
-    </row>
-    <row r="11" spans="1:9" s="120" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A11" s="117"/>
-      <c r="B11" s="121" t="s">
-        <v>173</v>
-      </c>
-      <c r="C11" s="118" t="s">
-        <v>179</v>
-      </c>
-      <c r="D11" s="135"/>
-      <c r="E11" s="136"/>
-      <c r="F11" s="136"/>
-      <c r="G11" s="136"/>
-      <c r="H11" s="123"/>
-      <c r="I11" s="119"/>
-    </row>
-    <row r="12" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="117"/>
-      <c r="B12" s="121" t="s">
-        <v>174</v>
-      </c>
-      <c r="C12" s="118"/>
-      <c r="D12" s="122"/>
-      <c r="E12" s="123"/>
-      <c r="F12" s="123"/>
-      <c r="G12" s="123"/>
-      <c r="H12" s="123"/>
-      <c r="I12" s="119"/>
-    </row>
-    <row r="13" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="117"/>
-      <c r="B13" s="121" t="s">
-        <v>175</v>
-      </c>
-      <c r="C13" s="118"/>
-      <c r="D13" s="122"/>
-      <c r="E13" s="123"/>
-      <c r="F13" s="123"/>
-      <c r="G13" s="123"/>
-      <c r="H13" s="123"/>
-      <c r="I13" s="119"/>
-    </row>
-    <row r="14" spans="1:9" s="120" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A14" s="117"/>
-      <c r="B14" s="124" t="s">
-        <v>176</v>
-      </c>
-      <c r="C14" s="118"/>
-      <c r="D14" s="122"/>
-      <c r="E14" s="123"/>
-      <c r="F14" s="123"/>
-      <c r="G14" s="123"/>
-      <c r="H14" s="123"/>
-      <c r="I14" s="119"/>
-    </row>
-    <row r="15" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="117"/>
-      <c r="B15" s="121" t="s">
-        <v>177</v>
-      </c>
-      <c r="C15" s="118"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
-      <c r="F15" s="123"/>
-      <c r="G15" s="123"/>
-      <c r="H15" s="123"/>
-      <c r="I15" s="119"/>
-    </row>
-    <row r="16" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="117"/>
-      <c r="B16" s="121" t="s">
-        <v>178</v>
-      </c>
-      <c r="C16" s="118"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
-      <c r="F16" s="123"/>
-      <c r="G16" s="123"/>
-      <c r="H16" s="123"/>
-      <c r="I16" s="119"/>
-    </row>
-    <row r="17" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="117"/>
-      <c r="B17" s="121" t="s">
-        <v>180</v>
-      </c>
-      <c r="C17" s="118" t="s">
-        <v>182</v>
-      </c>
-      <c r="D17" s="130"/>
-      <c r="E17" s="131"/>
-      <c r="F17" s="131"/>
-      <c r="G17" s="131"/>
-      <c r="H17" s="131"/>
-      <c r="I17" s="119"/>
-    </row>
-    <row r="18" spans="1:9" s="120" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="117"/>
-      <c r="B18" s="121" t="s">
-        <v>181</v>
-      </c>
-      <c r="C18" s="118" t="s">
-        <v>183</v>
-      </c>
-      <c r="D18" s="132"/>
-      <c r="E18" s="133"/>
-      <c r="F18" s="133"/>
-      <c r="G18" s="131"/>
-      <c r="H18" s="131"/>
-      <c r="I18" s="119"/>
-    </row>
-    <row r="19" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:9" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="33" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="34" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="35" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="36" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="37" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="38" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="39" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="40" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="41" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="42" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="43" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="44" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="45" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="46" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="47" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="48" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="65" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="66" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="67" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="68" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-    <row r="69" customFormat="1" ht="15" x14ac:dyDescent="0.2"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C1C4E25D-ABA5-41C3-BED8-BDADE1856557}">
-          <x14:formula1>
-            <xm:f>'Drop Down List Values'!$A$2:$A$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>H11</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5D77A5B3-DC21-4455-8579-74CE8C477205}">
-          <x14:formula1>
-            <xm:f>'Drop Down List Values'!$C$2:$C$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>H13</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{73E3C8C7-4C35-407D-BD90-B3CE9EDEF4AB}">
-          <x14:formula1>
-            <xm:f>'Drop Down List Values'!$B$2:$B$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>H12</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B2DC812E-574B-475E-A423-79EFE715328F}">
-          <x14:formula1>
-            <xm:f>'Drop Down List Values'!N1:N6</xm:f>
-          </x14:formula1>
-          <xm:sqref>D4:H4</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F8BFBD-18C1-4ED5-A02E-9841686C259E}">
   <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4128,7 +3477,7 @@
         <v>120</v>
       </c>
       <c r="N1" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
@@ -4169,10 +3518,10 @@
         <v>135</v>
       </c>
       <c r="M2" t="s">
-        <v>219</v>
+        <v>191</v>
       </c>
       <c r="N2" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
@@ -4213,10 +3562,10 @@
         <v>141</v>
       </c>
       <c r="M3" t="s">
-        <v>220</v>
+        <v>192</v>
       </c>
       <c r="N3" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -4257,10 +3606,10 @@
         <v>151</v>
       </c>
       <c r="M4" t="s">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="N4" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -4298,7 +3647,7 @@
         <v>144</v>
       </c>
       <c r="N5" t="s">
-        <v>190</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -4321,7 +3670,7 @@
         <v>159</v>
       </c>
       <c r="N6" t="s">
-        <v>191</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -4345,79 +3694,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
-      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
-      <Description>YVWEJ5DVYS2U-421999773-68</Description>
-    </_dlc_DocIdUrl>
-    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D4902BA52C7D94A994657A564808B2B" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4455a60d2ff5f5fcd8815d6d89b5b66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b541edd5-2552-480e-ada6-0e2c8d317108" xmlns:ns3="780ae317-08c5-4e10-af93-dd385a8384a9" xmlns:ns4="3146657c-56f4-4c0a-bb9c-a675121ac670" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1d01ecd782f081d5d944fa263943fc4" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="b541edd5-2552-480e-ada6-0e2c8d317108"/>
@@ -4616,23 +3892,100 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
+      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
+      <Description>YVWEJ5DVYS2U-421999773-68</Description>
+    </_dlc_DocIdUrl>
+    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
+    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
+    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4650,22 +4003,18 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
-    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
-    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Funeral Tracking number added for DCR
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F18E4E-07B4-5244-BD00-89625AC1620F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AE397D-B43E-E741-8D40-9EFD15E002FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="840" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
+    <workbookView xWindow="0" yWindow="1340" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
   <sheets>
     <sheet name="DCR" sheetId="4" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="217">
   <si>
     <t>Sections</t>
   </si>
@@ -778,6 +778,12 @@
   <si>
     <t>Funeral Home Director's identifier value</t>
   </si>
+  <si>
+    <t>Tracking Number: Funeral Home Case Number</t>
+  </si>
+  <si>
+    <t>A locally unique case number from the funeral home system.</t>
+  </si>
 </sst>
 </file>
 
@@ -786,7 +792,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -865,6 +871,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="22">
@@ -992,7 +1004,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1089,6 +1101,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1097,7 +1122,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1297,9 +1322,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1545,6 +1567,17 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1879,11 +1912,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU92"/>
+  <dimension ref="A1:AU93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
-    <col min="2" max="2" width="24.5" style="123" customWidth="1"/>
+    <col min="2" max="2" width="24.5" style="122" customWidth="1"/>
     <col min="3" max="3" width="39.1640625" style="58" customWidth="1"/>
     <col min="4" max="8" width="32.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
@@ -1894,7 +1927,7 @@
       <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="123" t="s">
+      <c r="B1" s="122" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="58" t="s">
@@ -1923,7 +1956,7 @@
       <c r="A2" s="46" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="122" t="s">
         <v>210</v>
       </c>
       <c r="C2" s="58" t="s">
@@ -1934,8 +1967,8 @@
       <c r="A3" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="124"/>
-      <c r="C3" s="81" t="s">
+      <c r="B3" s="123"/>
+      <c r="C3" s="80" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1943,7 +1976,7 @@
       <c r="A4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="125"/>
+      <c r="B4" s="124"/>
       <c r="C4" s="62" t="s">
         <v>12</v>
       </c>
@@ -1956,228 +1989,230 @@
     </row>
     <row r="5" spans="1:9" s="6" customFormat="1" ht="31" x14ac:dyDescent="0.3">
       <c r="A5" s="48"/>
-      <c r="B5" s="78" t="s">
+      <c r="B5" s="77" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="89"/>
+      <c r="G5" s="89"/>
+      <c r="H5" s="89"/>
       <c r="I5" s="5"/>
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A6" s="48"/>
-      <c r="B6" s="79" t="s">
+      <c r="B6" s="78" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="90"/>
-      <c r="E6" s="90"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
+      <c r="D6" s="89"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="89"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A7" s="49" t="s">
+    <row r="7" spans="1:9" s="6" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A7" s="48"/>
+      <c r="B7" s="139" t="s">
+        <v>215</v>
+      </c>
+      <c r="C7" s="140" t="s">
+        <v>216</v>
+      </c>
+      <c r="D7" s="89"/>
+      <c r="E7" s="89"/>
+      <c r="F7" s="89"/>
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" s="8" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A8" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="126"/>
-      <c r="C7" s="64" t="s">
+      <c r="B8" s="125"/>
+      <c r="C8" s="138" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:9" s="11" customFormat="1" ht="78" x14ac:dyDescent="0.3">
-      <c r="A8" s="50"/>
-      <c r="B8" s="59" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="65" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="91"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
-    </row>
-    <row r="9" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+    </row>
+    <row r="9" spans="1:9" s="11" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A9" s="50"/>
       <c r="B9" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="65" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="91"/>
+        <v>19</v>
+      </c>
+      <c r="C9" s="64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="90"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A10" s="50"/>
       <c r="B10" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="65" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="91"/>
+        <v>21</v>
+      </c>
+      <c r="C10" s="64" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="90"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="10"/>
     </row>
-    <row r="11" spans="1:9" s="11" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A11" s="50"/>
-      <c r="B11" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="65" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="91"/>
+      <c r="B11" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="90"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" s="11" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A12" s="50"/>
-      <c r="B12" s="59" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="65" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="91"/>
+      <c r="B12" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="64" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="90"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:9" s="11" customFormat="1" ht="65" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A13" s="50"/>
       <c r="B13" s="59" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="91"/>
+        <v>30</v>
+      </c>
+      <c r="C13" s="64" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="90"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" s="11" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A14" s="50"/>
       <c r="B14" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="65" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="93"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
+        <v>32</v>
+      </c>
+      <c r="C14" s="64" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="90"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" s="11" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A15" s="50"/>
       <c r="B15" s="59" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="65"/>
-      <c r="D15" s="91"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+        <v>34</v>
+      </c>
+      <c r="C15" s="64" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="92"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="50"/>
       <c r="B16" s="59" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="65" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="110"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="111"/>
+        <v>36</v>
+      </c>
+      <c r="C16" s="64"/>
+      <c r="D16" s="90"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
       <c r="I16" s="10"/>
     </row>
-    <row r="17" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" s="11" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A17" s="50"/>
       <c r="B17" s="59" t="s">
-        <v>169</v>
-      </c>
-      <c r="C17" s="65"/>
-      <c r="D17" s="91"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
+        <v>37</v>
+      </c>
+      <c r="C17" s="64" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="109"/>
+      <c r="E17" s="110"/>
+      <c r="F17" s="110"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
       <c r="I17" s="10"/>
     </row>
-    <row r="18" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="50"/>
       <c r="B18" s="59" t="s">
-        <v>170</v>
-      </c>
-      <c r="C18" s="65"/>
-      <c r="D18" s="91"/>
+        <v>169</v>
+      </c>
+      <c r="C18" s="64"/>
+      <c r="D18" s="90"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
       <c r="I18" s="10"/>
     </row>
-    <row r="19" spans="1:9" s="11" customFormat="1" ht="42" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A19" s="50"/>
       <c r="B19" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="65"/>
-      <c r="D19" s="91"/>
+        <v>170</v>
+      </c>
+      <c r="C19" s="64"/>
+      <c r="D19" s="90"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="11" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A20" s="50"/>
       <c r="B20" s="59" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="65"/>
-      <c r="D20" s="91"/>
+        <v>39</v>
+      </c>
+      <c r="C20" s="64"/>
+      <c r="D20" s="90"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -2187,100 +2222,98 @@
     <row r="21" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A21" s="50"/>
       <c r="B21" s="59" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="65"/>
-      <c r="D21" s="91"/>
+        <v>40</v>
+      </c>
+      <c r="C21" s="64"/>
+      <c r="D21" s="90"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
       <c r="I21" s="10"/>
     </row>
-    <row r="22" spans="1:9" s="13" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A22" s="75" t="s">
+    <row r="22" spans="1:9" s="11" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+      <c r="A22" s="50"/>
+      <c r="B22" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="64"/>
+      <c r="D22" s="90"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="10"/>
+    </row>
+    <row r="23" spans="1:9" s="13" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+      <c r="A23" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="128"/>
-      <c r="C22" s="66" t="s">
+      <c r="B23" s="127"/>
+      <c r="C23" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="92"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="92"/>
-      <c r="G22" s="92"/>
-      <c r="H22" s="92"/>
-      <c r="I22" s="92"/>
-    </row>
-    <row r="23" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="51"/>
-      <c r="B23" s="80" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="67" t="s">
-        <v>45</v>
-      </c>
-      <c r="D23" s="99"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="83"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="91"/>
+      <c r="H23" s="91"/>
+      <c r="I23" s="91"/>
     </row>
     <row r="24" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="51"/>
-      <c r="B24" s="80" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="67" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="95"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="84"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
+      <c r="B24" s="79" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="66" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="98"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="82"/>
+      <c r="H24" s="14"/>
       <c r="I24" s="15"/>
     </row>
     <row r="25" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="51"/>
-      <c r="B25" s="80" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25" s="67" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="96"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
+      <c r="B25" s="79" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="94"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
       <c r="I25" s="15"/>
     </row>
     <row r="26" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="51"/>
-      <c r="B26" s="80" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="67" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26" s="96"/>
+      <c r="B26" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="95"/>
       <c r="E26" s="18"/>
       <c r="F26" s="18"/>
       <c r="G26" s="18"/>
       <c r="H26" s="18"/>
       <c r="I26" s="15"/>
     </row>
-    <row r="27" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="51"/>
-      <c r="B27" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="67" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27" s="96"/>
+      <c r="B27" s="79" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="66" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="95"/>
       <c r="E27" s="18"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2289,13 +2322,13 @@
     </row>
     <row r="28" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A28" s="51"/>
-      <c r="B28" s="80" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28" s="67" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28" s="96"/>
+      <c r="B28" s="79" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="66" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" s="95"/>
       <c r="E28" s="18"/>
       <c r="F28" s="18"/>
       <c r="G28" s="18"/>
@@ -2304,13 +2337,13 @@
     </row>
     <row r="29" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A29" s="51"/>
-      <c r="B29" s="80" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="67" t="s">
-        <v>57</v>
-      </c>
-      <c r="D29" s="96"/>
+      <c r="B29" s="79" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="66" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="95"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -2319,161 +2352,163 @@
     </row>
     <row r="30" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
       <c r="A30" s="51"/>
-      <c r="B30" s="80" t="s">
+      <c r="B30" s="79" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="66" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="95"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="15"/>
+    </row>
+    <row r="31" spans="1:9" s="16" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+      <c r="A31" s="51"/>
+      <c r="B31" s="79" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="67" t="s">
+      <c r="C31" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="94"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15"/>
-    </row>
-    <row r="31" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A31" s="51"/>
-      <c r="B31" s="80" t="s">
+      <c r="D31" s="93"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="15"/>
+    </row>
+    <row r="32" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A32" s="51"/>
+      <c r="B32" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="67" t="s">
+      <c r="C32" s="66" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="96"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="15"/>
-    </row>
-    <row r="32" spans="1:9" s="16" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A32" s="51"/>
-      <c r="B32" s="60" t="s">
-        <v>62</v>
-      </c>
-      <c r="C32" s="67" t="s">
-        <v>63</v>
-      </c>
-      <c r="D32" s="97"/>
-      <c r="E32" s="19"/>
+      <c r="D32" s="95"/>
+      <c r="E32" s="18"/>
       <c r="F32" s="19"/>
       <c r="G32" s="19"/>
       <c r="H32" s="19"/>
       <c r="I32" s="15"/>
     </row>
-    <row r="33" spans="1:9" s="16" customFormat="1" ht="65" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" s="16" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A33" s="51"/>
       <c r="B33" s="60" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="67" t="s">
-        <v>66</v>
-      </c>
-      <c r="D33" s="98"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
+        <v>62</v>
+      </c>
+      <c r="C33" s="66" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="96"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
       <c r="I33" s="15"/>
     </row>
-    <row r="34" spans="1:9" s="16" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" s="16" customFormat="1" ht="65" x14ac:dyDescent="0.3">
       <c r="A34" s="51"/>
       <c r="B34" s="60" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="66" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="97"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="15"/>
+    </row>
+    <row r="35" spans="1:9" s="16" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+      <c r="A35" s="51"/>
+      <c r="B35" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="67" t="s">
+      <c r="C35" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="D34" s="100"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="85"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="15"/>
-    </row>
-    <row r="35" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="52"/>
-      <c r="B35" s="60" t="s">
+      <c r="D35" s="99"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="84"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="15"/>
+    </row>
+    <row r="36" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="52"/>
+      <c r="B36" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C36" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="96"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="22"/>
-    </row>
-    <row r="36" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A36" s="51"/>
-      <c r="B36" s="60" t="s">
-        <v>71</v>
-      </c>
-      <c r="C36" s="67" t="s">
-        <v>72</v>
-      </c>
-      <c r="D36" s="97"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="15"/>
+      <c r="D36" s="95"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="22"/>
     </row>
     <row r="37" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A37" s="51"/>
       <c r="B37" s="60" t="s">
-        <v>74</v>
-      </c>
-      <c r="C37" s="67" t="s">
-        <v>75</v>
-      </c>
-      <c r="D37" s="97"/>
+        <v>71</v>
+      </c>
+      <c r="C37" s="66" t="s">
+        <v>72</v>
+      </c>
+      <c r="D37" s="96"/>
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
       <c r="H37" s="19"/>
       <c r="I37" s="15"/>
     </row>
-    <row r="38" spans="1:9" s="25" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A38" s="76" t="s">
+    <row r="38" spans="1:9" s="16" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A38" s="51"/>
+      <c r="B38" s="60" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="66" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="96"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="15"/>
+    </row>
+    <row r="39" spans="1:9" s="25" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+      <c r="A39" s="75" t="s">
         <v>76</v>
       </c>
-      <c r="B38" s="129"/>
-      <c r="C38" s="68" t="s">
+      <c r="B39" s="128"/>
+      <c r="C39" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
-    </row>
-    <row r="39" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A39" s="53"/>
-      <c r="B39" s="77" t="s">
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
+    </row>
+    <row r="40" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A40" s="53"/>
+      <c r="B40" s="76" t="s">
         <v>171</v>
       </c>
-      <c r="C39" s="69" t="s">
+      <c r="C40" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="D39" s="102"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="27"/>
-    </row>
-    <row r="40" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="53"/>
-      <c r="B40" s="77" t="s">
-        <v>173</v>
-      </c>
-      <c r="C40" s="69"/>
-      <c r="D40" s="102"/>
+      <c r="D40" s="101"/>
       <c r="E40" s="26"/>
       <c r="F40" s="26"/>
       <c r="G40" s="26"/>
@@ -2482,393 +2517,355 @@
     </row>
     <row r="41" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="53"/>
-      <c r="B41" s="77" t="s">
-        <v>174</v>
-      </c>
-      <c r="C41" s="69"/>
-      <c r="D41" s="102"/>
+      <c r="B41" s="76" t="s">
+        <v>173</v>
+      </c>
+      <c r="C41" s="68"/>
+      <c r="D41" s="101"/>
       <c r="E41" s="26"/>
       <c r="F41" s="26"/>
       <c r="G41" s="26"/>
       <c r="H41" s="26"/>
       <c r="I41" s="27"/>
     </row>
-    <row r="42" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="53"/>
-      <c r="B42" s="77" t="s">
-        <v>175</v>
-      </c>
-      <c r="C42" s="69"/>
-      <c r="D42" s="102"/>
+      <c r="B42" s="76" t="s">
+        <v>174</v>
+      </c>
+      <c r="C42" s="68"/>
+      <c r="D42" s="101"/>
       <c r="E42" s="26"/>
       <c r="F42" s="26"/>
       <c r="G42" s="26"/>
       <c r="H42" s="26"/>
       <c r="I42" s="27"/>
     </row>
-    <row r="43" spans="1:9" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A43" s="53"/>
-      <c r="B43" s="77" t="s">
-        <v>176</v>
-      </c>
-      <c r="C43" s="69"/>
-      <c r="D43" s="102"/>
+      <c r="B43" s="76" t="s">
+        <v>175</v>
+      </c>
+      <c r="C43" s="68"/>
+      <c r="D43" s="101"/>
       <c r="E43" s="26"/>
       <c r="F43" s="26"/>
       <c r="G43" s="26"/>
       <c r="H43" s="26"/>
       <c r="I43" s="27"/>
     </row>
-    <row r="44" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A44" s="53"/>
-      <c r="B44" s="77" t="s">
-        <v>177</v>
-      </c>
-      <c r="C44" s="69"/>
-      <c r="D44" s="102"/>
+      <c r="B44" s="76" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44" s="68"/>
+      <c r="D44" s="101"/>
       <c r="E44" s="26"/>
       <c r="F44" s="26"/>
       <c r="G44" s="26"/>
       <c r="H44" s="26"/>
       <c r="I44" s="27"/>
     </row>
-    <row r="45" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="53"/>
-      <c r="B45" s="130" t="s">
+      <c r="B45" s="76" t="s">
+        <v>177</v>
+      </c>
+      <c r="C45" s="68"/>
+      <c r="D45" s="101"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="26"/>
+      <c r="H45" s="26"/>
+      <c r="I45" s="27"/>
+    </row>
+    <row r="46" spans="1:9" s="28" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A46" s="53"/>
+      <c r="B46" s="129" t="s">
         <v>178</v>
       </c>
-      <c r="C45" s="69" t="s">
+      <c r="C46" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="D45" s="102"/>
-      <c r="E45" s="112"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="112"/>
-      <c r="H45" s="112"/>
-      <c r="I45" s="27"/>
-    </row>
-    <row r="46" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="53"/>
-      <c r="B46" s="130" t="s">
-        <v>179</v>
-      </c>
-      <c r="C46" s="69"/>
-      <c r="D46" s="102"/>
-      <c r="E46" s="112"/>
+      <c r="D46" s="101"/>
+      <c r="E46" s="111"/>
       <c r="F46" s="26"/>
-      <c r="G46" s="112"/>
-      <c r="H46" s="112"/>
+      <c r="G46" s="111"/>
+      <c r="H46" s="111"/>
       <c r="I46" s="27"/>
     </row>
     <row r="47" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="53"/>
-      <c r="B47" s="130" t="s">
+      <c r="B47" s="129" t="s">
+        <v>179</v>
+      </c>
+      <c r="C47" s="68"/>
+      <c r="D47" s="101"/>
+      <c r="E47" s="111"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="111"/>
+      <c r="H47" s="111"/>
+      <c r="I47" s="27"/>
+    </row>
+    <row r="48" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="53"/>
+      <c r="B48" s="129" t="s">
         <v>180</v>
       </c>
-      <c r="C47" s="69"/>
-      <c r="D47" s="102"/>
-      <c r="E47" s="112"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="112"/>
-      <c r="H47" s="112"/>
-      <c r="I47" s="27"/>
-    </row>
-    <row r="48" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
-      <c r="A48" s="53"/>
-      <c r="B48" s="130" t="s">
+      <c r="C48" s="68"/>
+      <c r="D48" s="101"/>
+      <c r="E48" s="111"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="111"/>
+      <c r="H48" s="111"/>
+      <c r="I48" s="27"/>
+    </row>
+    <row r="49" spans="1:9" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.3">
+      <c r="A49" s="53"/>
+      <c r="B49" s="129" t="s">
         <v>181</v>
       </c>
-      <c r="C48" s="69"/>
-      <c r="D48" s="102"/>
-      <c r="E48" s="112"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="112"/>
-      <c r="H48" s="112"/>
-      <c r="I48" s="27"/>
-    </row>
-    <row r="49" spans="1:47" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A49" s="53"/>
-      <c r="B49" s="130" t="s">
+      <c r="C49" s="68"/>
+      <c r="D49" s="101"/>
+      <c r="E49" s="111"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="111"/>
+      <c r="H49" s="111"/>
+      <c r="I49" s="27"/>
+    </row>
+    <row r="50" spans="1:9" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+      <c r="A50" s="53"/>
+      <c r="B50" s="129" t="s">
         <v>182</v>
       </c>
-      <c r="C49" s="69"/>
-      <c r="D49" s="102"/>
-      <c r="E49" s="112"/>
-      <c r="F49" s="26"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="112"/>
-      <c r="I49" s="27"/>
-    </row>
-    <row r="50" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="53"/>
-      <c r="B50" s="130" t="s">
+      <c r="C50" s="68"/>
+      <c r="D50" s="101"/>
+      <c r="E50" s="111"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="111"/>
+      <c r="H50" s="111"/>
+      <c r="I50" s="27"/>
+    </row>
+    <row r="51" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="53"/>
+      <c r="B51" s="129" t="s">
         <v>183</v>
       </c>
-      <c r="C50" s="69"/>
-      <c r="D50" s="102"/>
-      <c r="E50" s="112"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="112"/>
-      <c r="H50" s="112"/>
-      <c r="I50" s="27"/>
-    </row>
-    <row r="51" spans="1:47" s="28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="53"/>
-      <c r="B51" s="77" t="s">
+      <c r="C51" s="68"/>
+      <c r="D51" s="101"/>
+      <c r="E51" s="111"/>
+      <c r="F51" s="26"/>
+      <c r="G51" s="111"/>
+      <c r="H51" s="111"/>
+      <c r="I51" s="27"/>
+    </row>
+    <row r="52" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="53"/>
+      <c r="B52" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="C51" s="69"/>
-      <c r="D51" s="102"/>
-      <c r="E51" s="102"/>
-      <c r="F51" s="102"/>
-      <c r="G51" s="102"/>
-      <c r="H51" s="102"/>
-      <c r="I51" s="27"/>
-    </row>
-    <row r="52" spans="1:47" s="28" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A52" s="53"/>
-      <c r="B52" s="77" t="s">
+      <c r="C52" s="68"/>
+      <c r="D52" s="101"/>
+      <c r="E52" s="101"/>
+      <c r="F52" s="101"/>
+      <c r="G52" s="101"/>
+      <c r="H52" s="101"/>
+      <c r="I52" s="27"/>
+    </row>
+    <row r="53" spans="1:9" s="28" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A53" s="53"/>
+      <c r="B53" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="C52" s="69" t="s">
+      <c r="C53" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="D52" s="102"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="26"/>
-      <c r="I52" s="27"/>
-    </row>
-    <row r="53" spans="1:47" s="31" customFormat="1" ht="65" x14ac:dyDescent="0.3">
-      <c r="A53" s="82" t="s">
+      <c r="D53" s="101"/>
+      <c r="E53" s="26"/>
+      <c r="F53" s="26"/>
+      <c r="G53" s="26"/>
+      <c r="H53" s="26"/>
+      <c r="I53" s="27"/>
+    </row>
+    <row r="54" spans="1:9" s="31" customFormat="1" ht="65" x14ac:dyDescent="0.3">
+      <c r="A54" s="81" t="s">
         <v>82</v>
       </c>
-      <c r="B53" s="131"/>
-      <c r="C53" s="70" t="s">
+      <c r="B54" s="130"/>
+      <c r="C54" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="D53" s="103"/>
-      <c r="E53" s="29"/>
-      <c r="F53" s="29"/>
-      <c r="G53" s="29"/>
-      <c r="H53" s="29"/>
-      <c r="I53" s="30"/>
-    </row>
-    <row r="54" spans="1:47" s="34" customFormat="1" ht="52" x14ac:dyDescent="0.3">
-      <c r="A54" s="54"/>
-      <c r="B54" s="132" t="s">
+      <c r="D54" s="102"/>
+      <c r="E54" s="29"/>
+      <c r="F54" s="29"/>
+      <c r="G54" s="29"/>
+      <c r="H54" s="29"/>
+      <c r="I54" s="30"/>
+    </row>
+    <row r="55" spans="1:9" s="34" customFormat="1" ht="52" x14ac:dyDescent="0.3">
+      <c r="A55" s="54"/>
+      <c r="B55" s="131" t="s">
         <v>84</v>
       </c>
-      <c r="C54" s="71" t="s">
+      <c r="C55" s="70" t="s">
         <v>85</v>
       </c>
-      <c r="D54" s="104"/>
-      <c r="E54" s="32"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="32"/>
-      <c r="H54" s="32"/>
-      <c r="I54" s="33"/>
-    </row>
-    <row r="55" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A55" s="54"/>
-      <c r="B55" s="132" t="s">
+      <c r="D55" s="103"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="32"/>
+      <c r="H55" s="32"/>
+      <c r="I55" s="33"/>
+    </row>
+    <row r="56" spans="1:9" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+      <c r="A56" s="54"/>
+      <c r="B56" s="131" t="s">
         <v>86</v>
       </c>
-      <c r="C55" s="71" t="s">
+      <c r="C56" s="70" t="s">
         <v>87</v>
       </c>
-      <c r="D55" s="105"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="35"/>
-      <c r="G55" s="35"/>
-      <c r="H55" s="35"/>
-      <c r="I55" s="33"/>
-    </row>
-    <row r="56" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A56" s="54"/>
-      <c r="B56" s="132" t="s">
+      <c r="D56" s="104"/>
+      <c r="E56" s="35"/>
+      <c r="F56" s="35"/>
+      <c r="G56" s="35"/>
+      <c r="H56" s="35"/>
+      <c r="I56" s="33"/>
+    </row>
+    <row r="57" spans="1:9" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A57" s="54"/>
+      <c r="B57" s="131" t="s">
         <v>88</v>
       </c>
-      <c r="C56" s="71" t="s">
+      <c r="C57" s="70" t="s">
         <v>89</v>
       </c>
-      <c r="D56" s="106"/>
-      <c r="E56" s="101"/>
-      <c r="F56" s="101"/>
-      <c r="G56" s="101"/>
-      <c r="H56" s="101"/>
-      <c r="I56" s="33"/>
-    </row>
-    <row r="57" spans="1:47" s="34" customFormat="1" ht="65" x14ac:dyDescent="0.3">
-      <c r="A57" s="54"/>
-      <c r="B57" s="132" t="s">
+      <c r="D57" s="105"/>
+      <c r="E57" s="100"/>
+      <c r="F57" s="100"/>
+      <c r="G57" s="100"/>
+      <c r="H57" s="100"/>
+      <c r="I57" s="33"/>
+    </row>
+    <row r="58" spans="1:9" s="34" customFormat="1" ht="65" x14ac:dyDescent="0.3">
+      <c r="A58" s="54"/>
+      <c r="B58" s="131" t="s">
         <v>91</v>
       </c>
-      <c r="C57" s="71" t="s">
+      <c r="C58" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="D57" s="107"/>
-      <c r="E57" s="36"/>
-      <c r="F57" s="36"/>
-      <c r="G57" s="36"/>
-      <c r="H57" s="36"/>
-      <c r="I57" s="33"/>
-    </row>
-    <row r="58" spans="1:47" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
-      <c r="A58" s="54"/>
-      <c r="B58" s="132" t="s">
+      <c r="D58" s="106"/>
+      <c r="E58" s="36"/>
+      <c r="F58" s="36"/>
+      <c r="G58" s="36"/>
+      <c r="H58" s="36"/>
+      <c r="I58" s="33"/>
+    </row>
+    <row r="59" spans="1:9" s="34" customFormat="1" ht="91" x14ac:dyDescent="0.3">
+      <c r="A59" s="54"/>
+      <c r="B59" s="131" t="s">
         <v>93</v>
       </c>
-      <c r="C58" s="71" t="s">
+      <c r="C59" s="70" t="s">
         <v>94</v>
       </c>
-      <c r="D58" s="105"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
-      <c r="G58" s="35"/>
-      <c r="H58" s="35"/>
-      <c r="I58" s="33"/>
-    </row>
-    <row r="59" spans="1:47" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
-      <c r="A59" s="54"/>
-      <c r="B59" s="132" t="s">
+      <c r="D59" s="104"/>
+      <c r="E59" s="35"/>
+      <c r="F59" s="35"/>
+      <c r="G59" s="35"/>
+      <c r="H59" s="35"/>
+      <c r="I59" s="33"/>
+    </row>
+    <row r="60" spans="1:9" s="34" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+      <c r="A60" s="54"/>
+      <c r="B60" s="131" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="71" t="s">
+      <c r="C60" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="D59" s="101"/>
-      <c r="E59" s="101"/>
-      <c r="F59" s="101"/>
-      <c r="G59" s="101"/>
-      <c r="H59" s="101"/>
-      <c r="I59" s="33"/>
-    </row>
-    <row r="60" spans="1:47" s="38" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A60" s="55" t="s">
+      <c r="D60" s="100"/>
+      <c r="E60" s="100"/>
+      <c r="F60" s="100"/>
+      <c r="G60" s="100"/>
+      <c r="H60" s="100"/>
+      <c r="I60" s="33"/>
+    </row>
+    <row r="61" spans="1:9" s="38" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A61" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="B60" s="133"/>
-      <c r="C60" s="72" t="s">
+      <c r="B61" s="132"/>
+      <c r="C61" s="71" t="s">
         <v>99</v>
       </c>
-      <c r="D60" s="37"/>
-      <c r="E60" s="37"/>
-      <c r="F60" s="37"/>
-      <c r="G60" s="37"/>
-      <c r="H60" s="37"/>
-      <c r="I60" s="37"/>
-    </row>
-    <row r="61" spans="1:47" s="41" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="56"/>
-      <c r="B61" s="134" t="s">
+      <c r="D61" s="37"/>
+      <c r="E61" s="37"/>
+      <c r="F61" s="37"/>
+      <c r="G61" s="37"/>
+      <c r="H61" s="37"/>
+      <c r="I61" s="37"/>
+    </row>
+    <row r="62" spans="1:9" s="41" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="56"/>
+      <c r="B62" s="133" t="s">
         <v>100</v>
       </c>
-      <c r="C61" s="73" t="s">
+      <c r="C62" s="72" t="s">
         <v>101</v>
       </c>
-      <c r="D61" s="108"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="39"/>
-      <c r="G61" s="39"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="40"/>
-    </row>
-    <row r="62" spans="1:47" s="41" customFormat="1" ht="26" x14ac:dyDescent="0.3">
-      <c r="A62" s="56"/>
-      <c r="B62" s="134" t="s">
-        <v>102</v>
-      </c>
-      <c r="C62" s="73" t="s">
-        <v>103</v>
-      </c>
-      <c r="D62" s="108"/>
+      <c r="D62" s="107"/>
       <c r="E62" s="39"/>
       <c r="F62" s="39"/>
       <c r="G62" s="39"/>
       <c r="H62" s="39"/>
       <c r="I62" s="40"/>
     </row>
-    <row r="63" spans="1:47" s="41" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" s="41" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A63" s="56"/>
-      <c r="B63" s="134" t="s">
+      <c r="B63" s="133" t="s">
+        <v>102</v>
+      </c>
+      <c r="C63" s="72" t="s">
+        <v>103</v>
+      </c>
+      <c r="D63" s="107"/>
+      <c r="E63" s="39"/>
+      <c r="F63" s="39"/>
+      <c r="G63" s="39"/>
+      <c r="H63" s="39"/>
+      <c r="I63" s="40"/>
+    </row>
+    <row r="64" spans="1:9" s="41" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+      <c r="A64" s="56"/>
+      <c r="B64" s="133" t="s">
         <v>104</v>
       </c>
-      <c r="C63" s="73" t="s">
+      <c r="C64" s="72" t="s">
         <v>105</v>
       </c>
-      <c r="D63" s="108"/>
-      <c r="E63" s="108"/>
-      <c r="F63" s="108"/>
-      <c r="G63" s="108"/>
-      <c r="H63" s="108"/>
-      <c r="I63" s="56"/>
-    </row>
-    <row r="64" spans="1:47" s="42" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A64" s="56"/>
-      <c r="B64" s="134" t="s">
+      <c r="D64" s="107"/>
+      <c r="E64" s="107"/>
+      <c r="F64" s="107"/>
+      <c r="G64" s="107"/>
+      <c r="H64" s="107"/>
+      <c r="I64" s="56"/>
+    </row>
+    <row r="65" spans="1:47" s="42" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+      <c r="A65" s="56"/>
+      <c r="B65" s="133" t="s">
         <v>106</v>
       </c>
-      <c r="C64" s="73" t="s">
+      <c r="C65" s="72" t="s">
         <v>107</v>
       </c>
-      <c r="D64" s="108"/>
-      <c r="E64" s="108"/>
-      <c r="F64" s="108"/>
-      <c r="G64" s="108"/>
-      <c r="H64" s="108"/>
-      <c r="I64" s="56"/>
-      <c r="J64" s="56"/>
-      <c r="K64" s="56"/>
-      <c r="L64" s="56"/>
-      <c r="M64" s="56"/>
-      <c r="N64" s="56"/>
-      <c r="O64" s="56"/>
-      <c r="P64" s="56"/>
-      <c r="Q64" s="56"/>
-      <c r="R64" s="56"/>
-      <c r="S64" s="56"/>
-      <c r="T64" s="56"/>
-      <c r="U64" s="56"/>
-      <c r="V64" s="56"/>
-      <c r="W64" s="56"/>
-      <c r="X64" s="56"/>
-      <c r="Y64" s="56"/>
-      <c r="Z64" s="56"/>
-      <c r="AA64" s="56"/>
-      <c r="AB64" s="56"/>
-      <c r="AC64" s="56"/>
-      <c r="AD64" s="56"/>
-      <c r="AE64" s="56"/>
-      <c r="AF64" s="56"/>
-      <c r="AG64" s="56"/>
-      <c r="AH64" s="56"/>
-      <c r="AI64" s="56"/>
-      <c r="AJ64" s="56"/>
-      <c r="AK64" s="56"/>
-      <c r="AL64" s="56"/>
-      <c r="AM64" s="56"/>
-      <c r="AN64" s="56"/>
-      <c r="AO64" s="56"/>
-      <c r="AP64" s="56"/>
-      <c r="AQ64" s="56"/>
-      <c r="AR64" s="56"/>
-      <c r="AS64" s="56"/>
-      <c r="AT64" s="56"/>
-      <c r="AU64" s="56"/>
-    </row>
-    <row r="65" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A65" s="56"/>
-      <c r="B65" s="134" t="s">
-        <v>108</v>
-      </c>
-      <c r="C65" s="73"/>
-      <c r="D65" s="108"/>
-      <c r="E65" s="108"/>
-      <c r="F65" s="108"/>
-      <c r="G65" s="108"/>
-      <c r="H65" s="108"/>
+      <c r="D65" s="107"/>
+      <c r="E65" s="107"/>
+      <c r="F65" s="107"/>
+      <c r="G65" s="107"/>
+      <c r="H65" s="107"/>
       <c r="I65" s="56"/>
       <c r="J65" s="56"/>
       <c r="K65" s="56"/>
@@ -2911,15 +2908,15 @@
     </row>
     <row r="66" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A66" s="56"/>
-      <c r="B66" s="134" t="s">
-        <v>109</v>
-      </c>
-      <c r="C66" s="73"/>
-      <c r="D66" s="108"/>
-      <c r="E66" s="108"/>
-      <c r="F66" s="108"/>
-      <c r="G66" s="108"/>
-      <c r="H66" s="108"/>
+      <c r="B66" s="133" t="s">
+        <v>108</v>
+      </c>
+      <c r="C66" s="72"/>
+      <c r="D66" s="107"/>
+      <c r="E66" s="107"/>
+      <c r="F66" s="107"/>
+      <c r="G66" s="107"/>
+      <c r="H66" s="107"/>
       <c r="I66" s="56"/>
       <c r="J66" s="56"/>
       <c r="K66" s="56"/>
@@ -2960,17 +2957,17 @@
       <c r="AT66" s="56"/>
       <c r="AU66" s="56"/>
     </row>
-    <row r="67" spans="1:47" s="45" customFormat="1" ht="56" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A67" s="56"/>
-      <c r="B67" s="134" t="s">
-        <v>110</v>
-      </c>
-      <c r="C67" s="73"/>
-      <c r="D67" s="108"/>
-      <c r="E67" s="108"/>
-      <c r="F67" s="108"/>
-      <c r="G67" s="108"/>
-      <c r="H67" s="108"/>
+      <c r="B67" s="133" t="s">
+        <v>109</v>
+      </c>
+      <c r="C67" s="72"/>
+      <c r="D67" s="107"/>
+      <c r="E67" s="107"/>
+      <c r="F67" s="107"/>
+      <c r="G67" s="107"/>
+      <c r="H67" s="107"/>
       <c r="I67" s="56"/>
       <c r="J67" s="56"/>
       <c r="K67" s="56"/>
@@ -3011,17 +3008,17 @@
       <c r="AT67" s="56"/>
       <c r="AU67" s="56"/>
     </row>
-    <row r="68" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:47" s="45" customFormat="1" ht="56" x14ac:dyDescent="0.3">
       <c r="A68" s="56"/>
-      <c r="B68" s="134" t="s">
-        <v>111</v>
-      </c>
-      <c r="C68" s="73"/>
-      <c r="D68" s="108"/>
-      <c r="E68" s="108"/>
-      <c r="F68" s="108"/>
-      <c r="G68" s="108"/>
-      <c r="H68" s="108"/>
+      <c r="B68" s="133" t="s">
+        <v>110</v>
+      </c>
+      <c r="C68" s="72"/>
+      <c r="D68" s="107"/>
+      <c r="E68" s="107"/>
+      <c r="F68" s="107"/>
+      <c r="G68" s="107"/>
+      <c r="H68" s="107"/>
       <c r="I68" s="56"/>
       <c r="J68" s="56"/>
       <c r="K68" s="56"/>
@@ -3062,140 +3059,176 @@
       <c r="AT68" s="56"/>
       <c r="AU68" s="56"/>
     </row>
-    <row r="69" spans="1:47" s="89" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="86" t="s">
+    <row r="69" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+      <c r="A69" s="56"/>
+      <c r="B69" s="133" t="s">
+        <v>111</v>
+      </c>
+      <c r="C69" s="72"/>
+      <c r="D69" s="107"/>
+      <c r="E69" s="107"/>
+      <c r="F69" s="107"/>
+      <c r="G69" s="107"/>
+      <c r="H69" s="107"/>
+      <c r="I69" s="56"/>
+      <c r="J69" s="56"/>
+      <c r="K69" s="56"/>
+      <c r="L69" s="56"/>
+      <c r="M69" s="56"/>
+      <c r="N69" s="56"/>
+      <c r="O69" s="56"/>
+      <c r="P69" s="56"/>
+      <c r="Q69" s="56"/>
+      <c r="R69" s="56"/>
+      <c r="S69" s="56"/>
+      <c r="T69" s="56"/>
+      <c r="U69" s="56"/>
+      <c r="V69" s="56"/>
+      <c r="W69" s="56"/>
+      <c r="X69" s="56"/>
+      <c r="Y69" s="56"/>
+      <c r="Z69" s="56"/>
+      <c r="AA69" s="56"/>
+      <c r="AB69" s="56"/>
+      <c r="AC69" s="56"/>
+      <c r="AD69" s="56"/>
+      <c r="AE69" s="56"/>
+      <c r="AF69" s="56"/>
+      <c r="AG69" s="56"/>
+      <c r="AH69" s="56"/>
+      <c r="AI69" s="56"/>
+      <c r="AJ69" s="56"/>
+      <c r="AK69" s="56"/>
+      <c r="AL69" s="56"/>
+      <c r="AM69" s="56"/>
+      <c r="AN69" s="56"/>
+      <c r="AO69" s="56"/>
+      <c r="AP69" s="56"/>
+      <c r="AQ69" s="56"/>
+      <c r="AR69" s="56"/>
+      <c r="AS69" s="56"/>
+      <c r="AT69" s="56"/>
+      <c r="AU69" s="56"/>
+    </row>
+    <row r="70" spans="1:47" s="88" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="85" t="s">
         <v>162</v>
       </c>
-      <c r="B69" s="135"/>
-      <c r="C69" s="87"/>
-      <c r="D69" s="88"/>
-      <c r="E69" s="88"/>
-      <c r="F69" s="88"/>
-      <c r="G69" s="88"/>
-      <c r="H69" s="88"/>
-      <c r="I69" s="88"/>
-    </row>
-    <row r="70" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A70" s="57"/>
-      <c r="B70" s="61" t="s">
-        <v>112</v>
-      </c>
-      <c r="C70" s="74" t="s">
-        <v>113</v>
-      </c>
-      <c r="D70" s="109"/>
-      <c r="E70" s="109"/>
-      <c r="F70" s="109"/>
-      <c r="G70" s="109"/>
-      <c r="H70" s="43"/>
-      <c r="I70" s="44"/>
+      <c r="B70" s="134"/>
+      <c r="C70" s="86"/>
+      <c r="D70" s="87"/>
+      <c r="E70" s="87"/>
+      <c r="F70" s="87"/>
+      <c r="G70" s="87"/>
+      <c r="H70" s="87"/>
+      <c r="I70" s="87"/>
     </row>
     <row r="71" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A71" s="57"/>
       <c r="B71" s="61" t="s">
-        <v>114</v>
-      </c>
-      <c r="C71" s="74"/>
-      <c r="D71" s="109"/>
-      <c r="E71" s="43"/>
-      <c r="F71" s="43"/>
-      <c r="G71" s="43"/>
+        <v>112</v>
+      </c>
+      <c r="C71" s="73" t="s">
+        <v>113</v>
+      </c>
+      <c r="D71" s="108"/>
+      <c r="E71" s="108"/>
+      <c r="F71" s="108"/>
+      <c r="G71" s="108"/>
       <c r="H71" s="43"/>
       <c r="I71" s="44"/>
     </row>
     <row r="72" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A72" s="57"/>
       <c r="B72" s="61" t="s">
-        <v>115</v>
-      </c>
-      <c r="C72" s="74"/>
-      <c r="D72" s="109"/>
+        <v>114</v>
+      </c>
+      <c r="C72" s="73"/>
+      <c r="D72" s="108"/>
       <c r="E72" s="43"/>
       <c r="F72" s="43"/>
       <c r="G72" s="43"/>
       <c r="H72" s="43"/>
       <c r="I72" s="44"/>
     </row>
-    <row r="73" spans="1:47" s="45" customFormat="1" ht="42" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A73" s="57"/>
       <c r="B73" s="61" t="s">
-        <v>116</v>
-      </c>
-      <c r="C73" s="74"/>
-      <c r="D73" s="109"/>
+        <v>115</v>
+      </c>
+      <c r="C73" s="73"/>
+      <c r="D73" s="108"/>
       <c r="E73" s="43"/>
       <c r="F73" s="43"/>
       <c r="G73" s="43"/>
       <c r="H73" s="43"/>
       <c r="I73" s="44"/>
     </row>
-    <row r="74" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:47" s="45" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A74" s="57"/>
       <c r="B74" s="61" t="s">
-        <v>117</v>
-      </c>
-      <c r="C74" s="74"/>
-      <c r="D74" s="109"/>
+        <v>116</v>
+      </c>
+      <c r="C74" s="73"/>
+      <c r="D74" s="108"/>
       <c r="E74" s="43"/>
       <c r="F74" s="43"/>
       <c r="G74" s="43"/>
       <c r="H74" s="43"/>
       <c r="I74" s="44"/>
     </row>
-    <row r="75" spans="1:47" s="45" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:47" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A75" s="57"/>
       <c r="B75" s="61" t="s">
-        <v>118</v>
-      </c>
-      <c r="C75" s="74" t="s">
-        <v>119</v>
-      </c>
-      <c r="D75" s="109"/>
+        <v>117</v>
+      </c>
+      <c r="C75" s="73"/>
+      <c r="D75" s="108"/>
       <c r="E75" s="43"/>
       <c r="F75" s="43"/>
       <c r="G75" s="43"/>
       <c r="H75" s="43"/>
       <c r="I75" s="44"/>
     </row>
-    <row r="76" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:47" s="45" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A76" s="57"/>
       <c r="B76" s="61" t="s">
-        <v>188</v>
-      </c>
-      <c r="C76" s="74" t="s">
-        <v>189</v>
-      </c>
-      <c r="D76" s="109"/>
+        <v>118</v>
+      </c>
+      <c r="C76" s="73" t="s">
+        <v>119</v>
+      </c>
+      <c r="D76" s="108"/>
       <c r="E76" s="43"/>
       <c r="F76" s="43"/>
       <c r="G76" s="43"/>
       <c r="H76" s="43"/>
       <c r="I76" s="44"/>
     </row>
-    <row r="77" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:47" s="45" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A77" s="57"/>
       <c r="B77" s="61" t="s">
-        <v>185</v>
-      </c>
-      <c r="C77" s="74" t="s">
-        <v>190</v>
-      </c>
-      <c r="D77" s="109"/>
+        <v>188</v>
+      </c>
+      <c r="C77" s="73" t="s">
+        <v>189</v>
+      </c>
+      <c r="D77" s="108"/>
       <c r="E77" s="43"/>
       <c r="F77" s="43"/>
       <c r="G77" s="43"/>
       <c r="H77" s="43"/>
       <c r="I77" s="44"/>
     </row>
-    <row r="78" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:47" s="45" customFormat="1" ht="39" x14ac:dyDescent="0.3">
       <c r="A78" s="57"/>
       <c r="B78" s="61" t="s">
-        <v>186</v>
-      </c>
-      <c r="C78" s="74" t="s">
-        <v>187</v>
-      </c>
-      <c r="D78" s="109"/>
+        <v>185</v>
+      </c>
+      <c r="C78" s="73" t="s">
+        <v>190</v>
+      </c>
+      <c r="D78" s="108"/>
       <c r="E78" s="43"/>
       <c r="F78" s="43"/>
       <c r="G78" s="43"/>
@@ -3205,196 +3238,211 @@
     <row r="79" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="57"/>
       <c r="B79" s="61" t="s">
-        <v>120</v>
-      </c>
-      <c r="C79" s="74" t="s">
-        <v>121</v>
-      </c>
-      <c r="D79" s="109"/>
+        <v>186</v>
+      </c>
+      <c r="C79" s="73" t="s">
+        <v>187</v>
+      </c>
+      <c r="D79" s="108"/>
       <c r="E79" s="43"/>
       <c r="F79" s="43"/>
       <c r="G79" s="43"/>
       <c r="H79" s="43"/>
       <c r="I79" s="44"/>
     </row>
-    <row r="80" spans="1:47" s="119" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="116" t="s">
+    <row r="80" spans="1:47" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="57"/>
+      <c r="B80" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="C80" s="73" t="s">
+        <v>121</v>
+      </c>
+      <c r="D80" s="108"/>
+      <c r="E80" s="43"/>
+      <c r="F80" s="43"/>
+      <c r="G80" s="43"/>
+      <c r="H80" s="43"/>
+      <c r="I80" s="44"/>
+    </row>
+    <row r="81" spans="1:9" s="118" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="115" t="s">
         <v>194</v>
       </c>
-      <c r="B80" s="136"/>
-      <c r="C80" s="117"/>
-      <c r="D80" s="118"/>
-      <c r="E80" s="118"/>
-      <c r="F80" s="118"/>
-      <c r="G80" s="118"/>
-      <c r="H80" s="118"/>
-      <c r="I80" s="118"/>
-    </row>
-    <row r="81" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="113"/>
-      <c r="B81" s="122" t="s">
+      <c r="B81" s="135"/>
+      <c r="C81" s="116"/>
+      <c r="D81" s="117"/>
+      <c r="E81" s="117"/>
+      <c r="F81" s="117"/>
+      <c r="G81" s="117"/>
+      <c r="H81" s="117"/>
+      <c r="I81" s="117"/>
+    </row>
+    <row r="82" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="112"/>
+      <c r="B82" s="121" t="s">
         <v>195</v>
       </c>
-      <c r="C81" s="120" t="s">
+      <c r="C82" s="119" t="s">
         <v>201</v>
       </c>
-      <c r="D81" s="121"/>
-      <c r="E81" s="121"/>
-      <c r="F81" s="121"/>
-      <c r="G81" s="121"/>
-      <c r="H81" s="121"/>
-      <c r="I81" s="114"/>
-    </row>
-    <row r="82" spans="1:9" s="115" customFormat="1" ht="31" x14ac:dyDescent="0.3">
-      <c r="A82" s="113"/>
-      <c r="B82" s="122" t="s">
+      <c r="D82" s="120"/>
+      <c r="E82" s="120"/>
+      <c r="F82" s="120"/>
+      <c r="G82" s="120"/>
+      <c r="H82" s="120"/>
+      <c r="I82" s="113"/>
+    </row>
+    <row r="83" spans="1:9" s="114" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A83" s="112"/>
+      <c r="B83" s="121" t="s">
         <v>206</v>
       </c>
-      <c r="C82" s="120" t="s">
+      <c r="C83" s="119" t="s">
         <v>207</v>
       </c>
-      <c r="D82" s="121"/>
-      <c r="E82" s="121"/>
-      <c r="F82" s="121"/>
-      <c r="G82" s="121"/>
-      <c r="H82" s="121"/>
-      <c r="I82" s="114"/>
-    </row>
-    <row r="83" spans="1:9" s="115" customFormat="1" ht="31" x14ac:dyDescent="0.3">
-      <c r="A83" s="113"/>
-      <c r="B83" s="122" t="s">
+      <c r="D83" s="120"/>
+      <c r="E83" s="120"/>
+      <c r="F83" s="120"/>
+      <c r="G83" s="120"/>
+      <c r="H83" s="120"/>
+      <c r="I83" s="113"/>
+    </row>
+    <row r="84" spans="1:9" s="114" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A84" s="112"/>
+      <c r="B84" s="121" t="s">
         <v>211</v>
       </c>
-      <c r="C83" s="120" t="s">
+      <c r="C84" s="119" t="s">
         <v>213</v>
       </c>
-      <c r="D83" s="121"/>
-      <c r="E83" s="121"/>
-      <c r="F83" s="121"/>
-      <c r="G83" s="121"/>
-      <c r="H83" s="121"/>
-      <c r="I83" s="114"/>
-    </row>
-    <row r="84" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="113"/>
-      <c r="B84" s="138" t="s">
+      <c r="D84" s="120"/>
+      <c r="E84" s="120"/>
+      <c r="F84" s="120"/>
+      <c r="G84" s="120"/>
+      <c r="H84" s="120"/>
+      <c r="I84" s="113"/>
+    </row>
+    <row r="85" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="112"/>
+      <c r="B85" s="137" t="s">
         <v>212</v>
       </c>
-      <c r="C84" s="115" t="s">
+      <c r="C85" s="114" t="s">
         <v>214</v>
       </c>
-      <c r="D84" s="121"/>
-      <c r="E84" s="121"/>
-      <c r="F84" s="121"/>
-      <c r="G84" s="121"/>
-      <c r="H84" s="121"/>
-      <c r="I84" s="114"/>
-    </row>
-    <row r="85" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="113"/>
-      <c r="B85" s="122" t="s">
+      <c r="D85" s="120"/>
+      <c r="E85" s="120"/>
+      <c r="F85" s="120"/>
+      <c r="G85" s="120"/>
+      <c r="H85" s="120"/>
+      <c r="I85" s="113"/>
+    </row>
+    <row r="86" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="112"/>
+      <c r="B86" s="121" t="s">
         <v>202</v>
       </c>
-      <c r="C85" s="120"/>
-      <c r="D85" s="121"/>
-      <c r="E85" s="121"/>
-      <c r="F85" s="121"/>
-      <c r="G85" s="121"/>
-      <c r="H85" s="121"/>
-      <c r="I85" s="114"/>
-    </row>
-    <row r="86" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="113"/>
-      <c r="B86" s="122" t="s">
+      <c r="C86" s="119"/>
+      <c r="D86" s="120"/>
+      <c r="E86" s="120"/>
+      <c r="F86" s="120"/>
+      <c r="G86" s="120"/>
+      <c r="H86" s="120"/>
+      <c r="I86" s="113"/>
+    </row>
+    <row r="87" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="112"/>
+      <c r="B87" s="121" t="s">
         <v>203</v>
       </c>
-      <c r="C86" s="120"/>
-      <c r="D86" s="121"/>
-      <c r="E86" s="121"/>
-      <c r="F86" s="121"/>
-      <c r="G86" s="121"/>
-      <c r="H86" s="121"/>
-      <c r="I86" s="114"/>
-    </row>
-    <row r="87" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="113"/>
-      <c r="B87" s="122" t="s">
+      <c r="C87" s="119"/>
+      <c r="D87" s="120"/>
+      <c r="E87" s="120"/>
+      <c r="F87" s="120"/>
+      <c r="G87" s="120"/>
+      <c r="H87" s="120"/>
+      <c r="I87" s="113"/>
+    </row>
+    <row r="88" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="112"/>
+      <c r="B88" s="121" t="s">
         <v>196</v>
       </c>
-      <c r="C87" s="120"/>
-      <c r="D87" s="121"/>
-      <c r="E87" s="121"/>
-      <c r="F87" s="121"/>
-      <c r="G87" s="121"/>
-      <c r="H87" s="121"/>
-      <c r="I87" s="114"/>
-    </row>
-    <row r="88" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="113"/>
-      <c r="B88" s="122" t="s">
+      <c r="C88" s="119"/>
+      <c r="D88" s="120"/>
+      <c r="E88" s="120"/>
+      <c r="F88" s="120"/>
+      <c r="G88" s="120"/>
+      <c r="H88" s="120"/>
+      <c r="I88" s="113"/>
+    </row>
+    <row r="89" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="112"/>
+      <c r="B89" s="121" t="s">
         <v>197</v>
       </c>
-      <c r="C88" s="120"/>
-      <c r="D88" s="121"/>
-      <c r="E88" s="121"/>
-      <c r="F88" s="121"/>
-      <c r="G88" s="121"/>
-      <c r="H88" s="121"/>
-      <c r="I88" s="114"/>
-    </row>
-    <row r="89" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="113"/>
-      <c r="B89" s="122" t="s">
+      <c r="C89" s="119"/>
+      <c r="D89" s="120"/>
+      <c r="E89" s="120"/>
+      <c r="F89" s="120"/>
+      <c r="G89" s="120"/>
+      <c r="H89" s="120"/>
+      <c r="I89" s="113"/>
+    </row>
+    <row r="90" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="112"/>
+      <c r="B90" s="121" t="s">
         <v>198</v>
       </c>
-      <c r="C89" s="120"/>
-      <c r="D89" s="121"/>
-      <c r="E89" s="121"/>
-      <c r="F89" s="121"/>
-      <c r="G89" s="121"/>
-      <c r="H89" s="121"/>
-      <c r="I89" s="114"/>
-    </row>
-    <row r="90" spans="1:9" s="115" customFormat="1" ht="45" x14ac:dyDescent="0.3">
-      <c r="A90" s="113"/>
-      <c r="B90" s="122" t="s">
+      <c r="C90" s="119"/>
+      <c r="D90" s="120"/>
+      <c r="E90" s="120"/>
+      <c r="F90" s="120"/>
+      <c r="G90" s="120"/>
+      <c r="H90" s="120"/>
+      <c r="I90" s="113"/>
+    </row>
+    <row r="91" spans="1:9" s="114" customFormat="1" ht="45" x14ac:dyDescent="0.3">
+      <c r="A91" s="112"/>
+      <c r="B91" s="121" t="s">
         <v>199</v>
       </c>
-      <c r="C90" s="120"/>
-      <c r="D90" s="121"/>
-      <c r="E90" s="121"/>
-      <c r="F90" s="121"/>
-      <c r="G90" s="121"/>
-      <c r="H90" s="121"/>
-      <c r="I90" s="114"/>
-    </row>
-    <row r="91" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="113"/>
-      <c r="B91" s="122" t="s">
+      <c r="C91" s="119"/>
+      <c r="D91" s="120"/>
+      <c r="E91" s="120"/>
+      <c r="F91" s="120"/>
+      <c r="G91" s="120"/>
+      <c r="H91" s="120"/>
+      <c r="I91" s="113"/>
+    </row>
+    <row r="92" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="112"/>
+      <c r="B92" s="121" t="s">
         <v>200</v>
       </c>
-      <c r="C91" s="120"/>
-      <c r="D91" s="121"/>
-      <c r="E91" s="121"/>
-      <c r="F91" s="121"/>
-      <c r="G91" s="121"/>
-      <c r="H91" s="121"/>
-      <c r="I91" s="114"/>
-    </row>
-    <row r="92" spans="1:9" s="115" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="113"/>
-      <c r="B92" s="137" t="s">
+      <c r="C92" s="119"/>
+      <c r="D92" s="120"/>
+      <c r="E92" s="120"/>
+      <c r="F92" s="120"/>
+      <c r="G92" s="120"/>
+      <c r="H92" s="120"/>
+      <c r="I92" s="113"/>
+    </row>
+    <row r="93" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="112"/>
+      <c r="B93" s="136" t="s">
         <v>204</v>
       </c>
-      <c r="C92" s="120" t="s">
+      <c r="C93" s="119" t="s">
         <v>205</v>
       </c>
-      <c r="D92" s="121"/>
-      <c r="E92" s="121"/>
-      <c r="F92" s="121"/>
-      <c r="G92" s="121"/>
-      <c r="H92" s="121"/>
-      <c r="I92" s="114"/>
+      <c r="D93" s="120"/>
+      <c r="E93" s="120"/>
+      <c r="F93" s="120"/>
+      <c r="G93" s="120"/>
+      <c r="H93" s="120"/>
+      <c r="I93" s="113"/>
     </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
@@ -3407,7 +3455,7 @@
           <x14:formula1>
             <xm:f>'Drop Down List Values'!$M$2:$M$5</xm:f>
           </x14:formula1>
-          <xm:sqref>D79:H79</xm:sqref>
+          <xm:sqref>D80:H80</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3694,6 +3742,65 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D4902BA52C7D94A994657A564808B2B" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4455a60d2ff5f5fcd8815d6d89b5b66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b541edd5-2552-480e-ada6-0e2c8d317108" xmlns:ns3="780ae317-08c5-4e10-af93-dd385a8384a9" xmlns:ns4="3146657c-56f4-4c0a-bb9c-a675121ac670" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1d01ecd782f081d5d944fa263943fc4" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="b541edd5-2552-480e-ada6-0e2c8d317108"/>
@@ -3892,7 +3999,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
@@ -3906,66 +4013,23 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0980278E-2A79-4F44-8623-FE545C304BE1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3985,7 +4049,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4001,20 +4065,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448710E8-BE9E-4C9E-A40A-0AC1DAE48E99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Funeral Home Email added
</commit_message>
<xml_diff>
--- a/import-templates/DCR-Template.xlsx
+++ b/import-templates/DCR-Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mc142/Documents/workspace/mortality-reporting/mdi-import/import-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AE397D-B43E-E741-8D40-9EFD15E002FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F41B22-6426-B840-8088-DF54D650C664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1340" windowWidth="34560" windowHeight="18960" xr2:uid="{7A50F290-1C75-487E-9806-F93553E4E7CC}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="219">
   <si>
     <t>Sections</t>
   </si>
@@ -783,6 +783,12 @@
   </si>
   <si>
     <t>A locally unique case number from the funeral home system.</t>
+  </si>
+  <si>
+    <t>Funeral Home: Email</t>
+  </si>
+  <si>
+    <t>Funeral Home Email Address</t>
   </si>
 </sst>
 </file>
@@ -1122,7 +1128,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -1578,6 +1584,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1912,7 +1921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD1DC7-E143-4CF5-BEA9-4DABBAFFC7B0}">
-  <dimension ref="A1:AU93"/>
+  <dimension ref="A1:AU94"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="21" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.33203125" style="46" customWidth="1"/>
@@ -3340,10 +3349,12 @@
     </row>
     <row r="86" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="112"/>
-      <c r="B86" s="121" t="s">
-        <v>202</v>
-      </c>
-      <c r="C86" s="119"/>
+      <c r="B86" s="137" t="s">
+        <v>217</v>
+      </c>
+      <c r="C86" s="141" t="s">
+        <v>218</v>
+      </c>
       <c r="D86" s="120"/>
       <c r="E86" s="120"/>
       <c r="F86" s="120"/>
@@ -3354,7 +3365,7 @@
     <row r="87" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="112"/>
       <c r="B87" s="121" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C87" s="119"/>
       <c r="D87" s="120"/>
@@ -3367,7 +3378,7 @@
     <row r="88" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A88" s="112"/>
       <c r="B88" s="121" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C88" s="119"/>
       <c r="D88" s="120"/>
@@ -3380,7 +3391,7 @@
     <row r="89" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="112"/>
       <c r="B89" s="121" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C89" s="119"/>
       <c r="D89" s="120"/>
@@ -3393,7 +3404,7 @@
     <row r="90" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A90" s="112"/>
       <c r="B90" s="121" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C90" s="119"/>
       <c r="D90" s="120"/>
@@ -3403,10 +3414,10 @@
       <c r="H90" s="120"/>
       <c r="I90" s="113"/>
     </row>
-    <row r="91" spans="1:9" s="114" customFormat="1" ht="45" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A91" s="112"/>
       <c r="B91" s="121" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C91" s="119"/>
       <c r="D91" s="120"/>
@@ -3416,10 +3427,10 @@
       <c r="H91" s="120"/>
       <c r="I91" s="113"/>
     </row>
-    <row r="92" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" s="114" customFormat="1" ht="45" x14ac:dyDescent="0.3">
       <c r="A92" s="112"/>
       <c r="B92" s="121" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C92" s="119"/>
       <c r="D92" s="120"/>
@@ -3431,18 +3442,31 @@
     </row>
     <row r="93" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="112"/>
-      <c r="B93" s="136" t="s">
-        <v>204</v>
-      </c>
-      <c r="C93" s="119" t="s">
-        <v>205</v>
-      </c>
+      <c r="B93" s="121" t="s">
+        <v>200</v>
+      </c>
+      <c r="C93" s="119"/>
       <c r="D93" s="120"/>
       <c r="E93" s="120"/>
       <c r="F93" s="120"/>
       <c r="G93" s="120"/>
       <c r="H93" s="120"/>
       <c r="I93" s="113"/>
+    </row>
+    <row r="94" spans="1:9" s="114" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="112"/>
+      <c r="B94" s="136" t="s">
+        <v>204</v>
+      </c>
+      <c r="C94" s="119" t="s">
+        <v>205</v>
+      </c>
+      <c r="D94" s="120"/>
+      <c r="E94" s="120"/>
+      <c r="F94" s="120"/>
+      <c r="G94" s="120"/>
+      <c r="H94" s="120"/>
+      <c r="I94" s="113"/>
     </row>
   </sheetData>
   <sheetProtection deleteColumns="0" selectLockedCells="1"/>
@@ -3751,53 +3775,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
+      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
+      <Description>YVWEJ5DVYS2U-421999773-68</Description>
+    </_dlc_DocIdUrl>
+    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4000,17 +3988,53 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">YVWEJ5DVYS2U-421999773-68</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="b541edd5-2552-480e-ada6-0e2c8d317108">
-      <Url>https://cdcpartners.sharepoint.com/sites/NCHS/nvssmodcop/_layouts/15/DocIdRedir.aspx?ID=YVWEJ5DVYS2U-421999773-68</Url>
-      <Description>YVWEJ5DVYS2U-421999773-68</Description>
-    </_dlc_DocIdUrl>
-    <ShareFileCreator xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-    <ShareFileCreated xmlns="780ae317-08c5-4e10-af93-dd385a8384a9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4022,9 +4046,19 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4050,19 +4084,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E3EF86-6C9E-4C22-A476-13DA012C68C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF0D7A6D-D78F-4048-9348-0B4289842B11}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="780ae317-08c5-4e10-af93-dd385a8384a9"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="b541edd5-2552-480e-ada6-0e2c8d317108"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3146657c-56f4-4c0a-bb9c-a675121ac670"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>